<commit_message>
Cobertura por simulación (en progreso): sondas de situación y jugadora automática
tools/cobertura.js le pregunta al juego qué reacciona en cada momento × lugar × cómo anda Ana ×
quién está, y una jugadora automática juega N días persiguiendo las metas del cuaderno.
tools/momentos.js: los momentos de la historia, compartidos con la planilla.
El planificador ya no se cae si recibe un objetivo que no puede perseguir (lo encontró la
jugadora automática).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VY3w9XmL1TrbHxLtQe81Lv
</commit_message>
<xml_diff>
--- a/planilla/avonlea.xlsx
+++ b/planilla/avonlea.xlsx
@@ -22,7 +22,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Frases'!$A$1:$J$2000</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cobertura'!$A$1:$E$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cobertura'!$A$1:$E$111</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Personas'!$A$1:$H$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Escenas'!$A$1:$Q$164</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Noticias'!$A$1:$K$14</definedName>
@@ -590,7 +590,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generada el 2026-10-16 06:50 desde los datos del juego (node tools/planilla.js).</t>
+          <t>Generada el 2026-10-16 07:00 desde los datos del juego (node tools/planilla.js).</t>
         </is>
       </c>
     </row>
@@ -30334,7 +30334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -30379,22 +30379,22 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>Noticias</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>«ana_lengua»: la niña de los Cuthbert tiene una lengua, pero buen corazón</t>
+          <t>Ana en camisón en la tienda de Lawson</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>nadie reacciona a ella (solo se cuenta)</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Lawson, la Sra. Pye)</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>una escena o una frase con «sabe:quien:ana_lengua» (alguien que se entera y hace o dice algo)</t>
+          <t>una escena con «si: ana:camison» (o la hora), y «ve:quien» o «en: quien=tl»</t>
         </is>
       </c>
     </row>
@@ -30406,76 +30406,76 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Noticias</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>«ana_ofendio_lynde»: la niña de los Cuthbert le dijo vieja chismosa a la Sra. Lynde</t>
+          <t>Ana en camisón en la escuela</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>nadie reacciona a ella (solo se cuenta)</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Phillips, la Srta. Stacy)</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>una escena o una frase con «sabe:quien:ana_ofendio_lynde» (alguien que se entera y hace o dice algo)</t>
+          <t>una escena con «si: ana:camison» (o la hora), y «ve:quien» o «en: quien=es»</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Noticias</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Ana en camisón en la casa del Sr. Harrison</t>
+          <t>«ana_lengua»: la niña de los Cuthbert tiene una lengua, pero buen corazón</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie reacciona a ella (solo se cuenta)</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>una escena con «si: ana:camison» (o la hora) y «en: …=hh»</t>
+          <t>una escena o una frase con «sabe:quien:ana_lengua» (alguien que se entera y hace o dice algo)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Noticias</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Ana en camisón en la tienda de Lawson</t>
+          <t>«ana_ofendio_lynde»: la niña de los Cuthbert le dijo vieja chismosa a la Sra. Lynde</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie reacciona a ella (solo se cuenta)</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>una escena con «si: ana:camison» (o la hora) y «en: …=tl»</t>
+          <t>una escena o una frase con «sabe:quien:ana_ofendio_lynde» (alguien que se entera y hace o dice algo)</t>
         </is>
       </c>
     </row>
@@ -30487,22 +30487,22 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Ana en camisón en la escuela</t>
+          <t>Ana en camisón en La Cuesta del Huerto</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie reacciona, en ningún momento (estaban: Mary Joe, el Sr. Barry, la Sra. Barry)</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>una escena con «si: ana:camison» (o la hora) y «en: …=es»</t>
+          <t>una escena con «si: ana:camison» (o la hora), y «ve:quien» o «en: quien=os»</t>
         </is>
       </c>
     </row>
@@ -30514,22 +30514,22 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Ana en camisón en la iglesia</t>
+          <t>Ana en camisón en la casa del Sr. Harrison</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Harrison)</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>una escena con «si: ana:camison» (o la hora) y «en: …=ig»</t>
+          <t>una escena con «si: ana:camison» (o la hora), y «ve:quien» o «en: quien=hh»</t>
         </is>
       </c>
     </row>
@@ -30541,7 +30541,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -30551,12 +30551,12 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie reacciona, en ningún momento (estaban: el reverendo Allan, la Sra. Allan)</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>una escena con «si: ana:camison» (o la hora) y «en: …=cp»</t>
+          <t>una escena con «si: ana:camison» (o la hora), y «ve:quien» o «en: quien=cp»</t>
         </is>
       </c>
     </row>
@@ -30568,22 +30568,22 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Ana en camisón en afuera (los caminos, la aldea)</t>
+          <t>Ana sin sombrero en Tejas Verdes</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie reacciona, en ningún momento (estaban: Marilla, Matthew, la Sra. Lynde)</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>una escena con «si: ana:camison» (o la hora) y «en: …=out»</t>
+          <t>una escena con «si: ana:sin_sombrero» (o la hora), y «ve:quien» o «en: quien=gg»</t>
         </is>
       </c>
     </row>
@@ -30595,22 +30595,22 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Ana sin sombrero en afuera (los caminos, la aldea)</t>
+          <t>Ana sin sombrero en La Cuesta del Huerto</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie reacciona, en ningún momento (estaban: Mary Joe, el Sr. Barry, la Sra. Barry)</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>una escena con «si: ana:sin_sombrero» (o la hora) y «en: …=out»</t>
+          <t>una escena con «si: ana:sin_sombrero» (o la hora), y «ve:quien» o «en: quien=os»</t>
         </is>
       </c>
     </row>
@@ -30622,22 +30622,22 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Ana sin sombrero en la iglesia</t>
+          <t>Ana sin sombrero en la Hondonada (Sra. Lynde)</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie reacciona, en ningún momento (estaban: Thomas Lynde, la Sra. Lynde)</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>una escena con «si: ana:sin_sombrero» (o la hora) y «en: …=ig»</t>
+          <t>una escena con «si: ana:sin_sombrero» (o la hora), y «ve:quien» o «en: quien=rl»</t>
         </is>
       </c>
     </row>
@@ -30649,22 +30649,22 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Ana sin sombrero en la escuela</t>
+          <t>Ana sin sombrero en la casa del Sr. Harrison</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Harrison)</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>una escena con «si: ana:sin_sombrero» (o la hora) y «en: …=es»</t>
+          <t>una escena con «si: ana:sin_sombrero» (o la hora), y «ve:quien» o «en: quien=hh»</t>
         </is>
       </c>
     </row>
@@ -30676,22 +30676,22 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Ana de noche en afuera (los caminos, la aldea)</t>
+          <t>Ana sin sombrero en la tienda de Lawson</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Lawson, la Sra. Pye)</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>una escena de noche (hora:21-26) en out</t>
+          <t>una escena con «si: ana:sin_sombrero» (o la hora), y «ve:quien» o «en: quien=tl»</t>
         </is>
       </c>
     </row>
@@ -30703,22 +30703,22 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Quién la ve en camisón</t>
+          <t>Ana sin sombrero en la escuela</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>no reaccionan: Matthew, Diana, el Sr. Harrison, el Sr. Shearer</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Phillips, la Srta. Stacy)</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>una escena «si: ana:camison, ve:quien» para cada uno</t>
+          <t>una escena con «si: ana:sin_sombrero» (o la hora), y «ve:quien» o «en: quien=es»</t>
         </is>
       </c>
     </row>
@@ -30730,22 +30730,22 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Frases</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Gertie Pye</t>
+          <t>Ana sin sombrero en la iglesia</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>no tiene qué decir: Día 2 (sin conocerla), Día 2 (conociéndola), Día 4 (sin conocerla), Día 4 (conociéndola), Día 16 (sin conocerla), Día 16 (conociéndola)…</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Bell, el reverendo Allan, la Sra. Allan, la Sra. Lynde, la Sra. Pye)</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>frases para esos momentos (hoja «Huecos»)</t>
+          <t>una escena con «si: ana:sin_sombrero» (o la hora), y «ve:quien» o «en: quien=ig»</t>
         </is>
       </c>
     </row>
@@ -30757,22 +30757,22 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Frases</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Jane Andrews</t>
+          <t>Ana sin sombrero en la casa parroquial</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>no tiene qué decir: Día 2 (sin conocerla), Día 4 (sin conocerla), Día 16 (sin conocerla), Día 20 (sin conocerla)</t>
+          <t>nadie reacciona, en ningún momento (estaban: el reverendo Allan, la Sra. Allan)</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>frases para esos momentos (hoja «Huecos»)</t>
+          <t>una escena con «si: ana:sin_sombrero» (o la hora), y «ve:quien» o «en: quien=cp»</t>
         </is>
       </c>
     </row>
@@ -30784,22 +30784,22 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Frases</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Charlie Sloane</t>
+          <t>Ana sin sombrero en la aldea (afuera)</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>no tiene qué decir: Día 2 (sin conocerla), Día 4 (sin conocerla), Día 16 (sin conocerla), Día 20 (sin conocerla), Día 33 (sin conocerla), Día 45 (sin conocerla)…</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Harrison, el Sr. Lawson, la Sra. Barry, la Sra. Lynde, la Sra. Pye, v0)</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>frases para esos momentos (hoja «Huecos»)</t>
+          <t>una escena con «si: ana:sin_sombrero» (o la hora), y «ve:quien» o «en: quien=out»</t>
         </is>
       </c>
     </row>
@@ -30811,22 +30811,22 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Frases</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Cecily King</t>
+          <t>Quién ve a Ana en camisón y no dice nada</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>no tiene qué decir: Día 2 (sin conocerla), Día 2 (conociéndola), Día 4 (sin conocerla), Día 4 (conociéndola), Día 16 (sin conocerla), Día 16 (conociéndola)…</t>
+          <t>Mary Joe, Matthew, Thomas Lynde, el Sr. Barry, el Sr. Bell, el Sr. Harrison, el Sr. Lawson, el Sr. Phillips, el reverendo Allan, la Sra. Allan, la Sra. Barry, la Sra. Pye, la Srta. Stacy, v0</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>frases para esos momentos (hoja «Huecos»)</t>
+          <t>una escena «si: ana:camison, ve:quien» (o una frase con [ana:camison])</t>
         </is>
       </c>
     </row>
@@ -30843,12 +30843,12 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Minnie May Barry</t>
+          <t>Gertie Pye</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>no tiene qué decir: Día 2 (sin conocerla), Día 4 (sin conocerla), Día 16 (sin conocerla), Día 20 (sin conocerla), Día 33 (sin conocerla), Día 45 (sin conocerla)…</t>
+          <t>no tiene qué decir: Día 2 (sin conocerla), Día 2 (conociéndola), Día 4 (sin conocerla), Día 4 (conociéndola), Día 16 (sin conocerla), Día 16 (conociéndola)…</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -30870,12 +30870,12 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Carrie Sloane</t>
+          <t>Jane Andrews</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>no tiene qué decir: Día 2 (sin conocerla), Día 2 (conociéndola), Día 4 (sin conocerla), Día 4 (conociéndola), Día 16 (sin conocerla), Día 16 (conociéndola)…</t>
+          <t>no tiene qué decir: Día 2 (sin conocerla), Día 4 (sin conocerla), Día 16 (sin conocerla), Día 20 (sin conocerla)</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -30897,12 +30897,12 @@
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>la Srta. Josephine Barry</t>
+          <t>Charlie Sloane</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>no tiene qué decir: Día 45 (sin conocerla), Día 45 (conociéndola)</t>
+          <t>no tiene qué decir: Día 2 (sin conocerla), Día 4 (sin conocerla), Día 16 (sin conocerla), Día 20 (sin conocerla), Día 33 (sin conocerla), Día 45 (sin conocerla)…</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -30919,22 +30919,22 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Metas</t>
+          <t>Frases</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>«perdon_barry»</t>
+          <t>Cecily King</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>nadie le sugiere a Ana hacerla (sin guiño)</t>
+          <t>no tiene qué decir: Día 2 (sin conocerla), Día 2 (conociéndola), Día 4 (sin conocerla), Día 4 (conociéndola), Día 16 (sin conocerla), Día 16 (conociéndola)…</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>«guiño quien: …» en src/datos/cuaderno.txt</t>
+          <t>frases para esos momentos (hoja «Huecos»)</t>
         </is>
       </c>
     </row>
@@ -30946,22 +30946,22 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Metas</t>
+          <t>Frases</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>«carta»</t>
+          <t>Minnie May Barry</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>nadie le sugiere a Ana hacerla (sin guiño)</t>
+          <t>no tiene qué decir: Día 2 (sin conocerla), Día 4 (sin conocerla), Día 16 (sin conocerla), Día 20 (sin conocerla), Día 33 (sin conocerla), Día 45 (sin conocerla)…</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>«guiño quien: …» en src/datos/cuaderno.txt</t>
+          <t>frases para esos momentos (hoja «Huecos»)</t>
         </is>
       </c>
     </row>
@@ -30973,22 +30973,22 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Metas</t>
+          <t>Frases</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>«sala»</t>
+          <t>Carrie Sloane</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>nadie le sugiere a Ana hacerla (sin guiño)</t>
+          <t>no tiene qué decir: Día 2 (sin conocerla), Día 2 (conociéndola), Día 4 (sin conocerla), Día 4 (conociéndola), Día 16 (sin conocerla), Día 16 (conociéndola)…</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>«guiño quien: …» en src/datos/cuaderno.txt</t>
+          <t>frases para esos momentos (hoja «Huecos»)</t>
         </is>
       </c>
     </row>
@@ -31000,22 +31000,22 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Metas</t>
+          <t>Frases</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>«sombrero»</t>
+          <t>la Srta. Josephine Barry</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>nadie le sugiere a Ana hacerla (sin guiño)</t>
+          <t>no tiene qué decir: Día 45 (sin conocerla), Día 45 (conociéndola)</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>«guiño quien: …» en src/datos/cuaderno.txt</t>
+          <t>frases para esos momentos (hoja «Huecos»)</t>
         </is>
       </c>
     </row>
@@ -31032,7 +31032,7 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>«tinte»</t>
+          <t>«perdon_barry»</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -31059,7 +31059,7 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>«pelo_corto»</t>
+          <t>«carta»</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
@@ -31086,7 +31086,7 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>«techo»</t>
+          <t>«sala»</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -31103,108 +31103,108 @@
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>media</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Metas</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Ana de noche en La Cuesta del Huerto (los Barry)</t>
+          <t>«sombrero»</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie le sugiere a Ana hacerla (sin guiño)</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>una escena de noche (hora:21-26) en os</t>
+          <t>«guiño quien: …» en src/datos/cuaderno.txt</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>media</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Metas</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Ana de noche en la Hondonada (la Sra. Lynde)</t>
+          <t>«tinte»</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie le sugiere a Ana hacerla (sin guiño)</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>una escena de noche (hora:21-26) en rl</t>
+          <t>«guiño quien: …» en src/datos/cuaderno.txt</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>media</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Ana y los lugares</t>
+          <t>Metas</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Ana de noche en la casa del Sr. Harrison</t>
+          <t>«pelo_corto»</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>ninguna escena reacciona</t>
+          <t>nadie le sugiere a Ana hacerla (sin guiño)</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>una escena de noche (hora:21-26) en hh</t>
+          <t>«guiño quien: …» en src/datos/cuaderno.txt</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>baja</t>
+          <t>media</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Noticias</t>
+          <t>Metas</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>«huerfano»: los Cuthbert van a traer un niño del orfanato</t>
+          <t>«techo»</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
+          <t>nadie le sugiere a Ana hacerla (sin guiño)</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>una escena o una frase con «sabe:quien:huerfano» (alguien que se entera y hace o dice algo)</t>
+          <t>«guiño quien: …» en src/datos/cuaderno.txt</t>
         </is>
       </c>
     </row>
@@ -31216,22 +31216,22 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Noticias</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>«cerdo_pye»: a los Pye se les escapó otra vez el cerdo</t>
+          <t>Ana de noche en Tejas Verdes</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
+          <t>nadie reacciona, en ningún momento (estaban: Marilla, Matthew, la Sra. Lynde)</t>
         </is>
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>una escena o una frase con «sabe:quien:cerdo_pye» (alguien que se entera y hace o dice algo)</t>
+          <t>una escena de noche (hora:21-26) con quien esté</t>
         </is>
       </c>
     </row>
@@ -31243,22 +31243,22 @@
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Noticias</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>«maestra_plumas»: la maestra nueva usa sombrero con plumas</t>
+          <t>Ana de noche en La Cuesta del Huerto</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
+          <t>nadie reacciona, en ningún momento (estaban: Mary Joe, el Sr. Barry, la Sra. Barry)</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>una escena o una frase con «sabe:quien:maestra_plumas» (alguien que se entera y hace o dice algo)</t>
+          <t>una escena de noche (hora:21-26) con quien esté</t>
         </is>
       </c>
     </row>
@@ -31270,22 +31270,22 @@
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Noticias</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>«loro_harrison»: el loro del Sr. Harrison dice cosas terribles</t>
+          <t>Ana de noche en la Hondonada (Sra. Lynde)</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
+          <t>nadie reacciona, en ningún momento (estaban: Thomas Lynde, la Sra. Lynde)</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>una escena o una frase con «sabe:quien:loro_harrison» (alguien que se entera y hace o dice algo)</t>
+          <t>una escena de noche (hora:21-26) con quien esté</t>
         </is>
       </c>
     </row>
@@ -31297,22 +31297,22 @@
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Noticias</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>«rastrillo_matthew»: Matthew Cuthbert compró un rastrillo en invierno</t>
+          <t>Ana de noche en la casa del Sr. Harrison</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Harrison)</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>una escena o una frase con «sabe:quien:rastrillo_matthew» (alguien que se entera y hace o dice algo)</t>
+          <t>una escena de noche (hora:21-26) con quien esté</t>
         </is>
       </c>
     </row>
@@ -31324,22 +31324,22 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Noticias</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>«ana_lengua»</t>
+          <t>Ana de noche en la tienda de Lawson</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>es de Ana y no tiene versión exagerada</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Lawson, la Sra. Pye)</t>
         </is>
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>una línea «exagerada:» (los chismosos la agrandan)</t>
+          <t>una escena de noche (hora:21-26) con quien esté</t>
         </is>
       </c>
     </row>
@@ -31351,22 +31351,22 @@
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Noticias</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>«pastor_nuevo»: llegó un pastor nuevo, el Sr. Allan, con su esposa</t>
+          <t>Ana de noche en la escuela</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Phillips, la Srta. Stacy)</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>una escena o una frase con «sabe:quien:pastor_nuevo» (alguien que se entera y hace o dice algo)</t>
+          <t>una escena de noche (hora:21-26) con quien esté</t>
         </is>
       </c>
     </row>
@@ -31378,22 +31378,22 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>Noticias</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>«tia_josephine»: la tía Josephine de los Barry vino de Charlottetown</t>
+          <t>Ana de noche en la iglesia</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Bell, el reverendo Allan, la Sra. Allan, la Sra. Lynde, la Sra. Pye)</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>una escena o una frase con «sabe:quien:tia_josephine» (alguien que se entera y hace o dice algo)</t>
+          <t>una escena de noche (hora:21-26) con quien esté</t>
         </is>
       </c>
     </row>
@@ -31405,22 +31405,22 @@
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Noticias</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>«se_va_phillips»: el Sr. Phillips se va de la escuela de Avonlea</t>
+          <t>Ana de noche en la casa parroquial</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
+          <t>nadie reacciona, en ningún momento (estaban: el reverendo Allan, la Sra. Allan)</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>una escena o una frase con «sabe:quien:se_va_phillips» (alguien que se entera y hace o dice algo)</t>
+          <t>una escena de noche (hora:21-26) con quien esté</t>
         </is>
       </c>
     </row>
@@ -31432,22 +31432,22 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>Llegadas</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Prissy Andrews se va</t>
+          <t>Ana de noche en la aldea (afuera)</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>nadie lo nota</t>
+          <t>nadie reacciona, en ningún momento (estaban: el Sr. Harrison, el Sr. Lawson, la Sra. Barry, la Sra. Lynde, la Sra. Pye, v0)</t>
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr">
         <is>
-          <t>una noticia o una escena con «hecho:se_fue_prissy»</t>
+          <t>una escena de noche (hora:21-26) con quien esté</t>
         </is>
       </c>
     </row>
@@ -31459,22 +31459,22 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>Llegadas</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>el buhonero llega (de visita)</t>
+          <t>Ana en camisón: ella misma no lo nota</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>nadie lo nota (solo queda en el diario)</t>
+          <t>en Tejas Verdes, La Cuesta del Huerto, la Hondonada (Sra. Lynde), la casa del Sr. Harrison, la tienda de Lawson, la escuela, la iglesia, la casa parroquial, la aldea (afuera)</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>una noticia «saben si hecho:llego_buhonero: …» o una escena «si: hecho:llego_buhonero»</t>
+          <t>un comentario de Ana con «si: ana:camison»</t>
         </is>
       </c>
     </row>
@@ -31486,22 +31486,22 @@
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>Llegadas</t>
+          <t>Situaciones</t>
         </is>
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>una veraneante del hotel llega (de visita)</t>
+          <t>Ana sin sombrero: ella misma no lo nota</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>nadie lo nota (solo queda en el diario)</t>
+          <t>en Tejas Verdes, La Cuesta del Huerto, la Hondonada (Sra. Lynde), la casa del Sr. Harrison, la tienda de Lawson, la escuela, la iglesia, la casa parroquial, la aldea (afuera)</t>
         </is>
       </c>
       <c r="E43" s="11" t="inlineStr">
         <is>
-          <t>una noticia «saben si hecho:llego_veraneante: …» o una escena «si: hecho:llego_veraneante»</t>
+          <t>un comentario de Ana con «si: ana:sin_sombrero»</t>
         </is>
       </c>
     </row>
@@ -31513,22 +31513,22 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Exploración</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Presentación propia (cómo se presenta la primera vez)</t>
+          <t>70 escena(s) que no pasaron en 4 días</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>32 usan la de siempre: Diana, el Sr. Shearer, el buhonero, el Sr. Phillips, el reverendo Allan, la Sra. Allan, el Sr. Lawson, el herrero, el editor de La Crónica, la Srta. Hetty King, Olivia King, Jasper Dale, Alec King, Janet King…</t>
+          <t>les falta: Ana no va en la calesa por el camino</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>«presentacion» en personajes.json, o «presenta» en src/js/56-gente-de-avonlea.js, con su voz</t>
+          <t>ej.: avenida, newbridge, avenida_petalos, avenida_paso</t>
         </is>
       </c>
     </row>
@@ -31540,22 +31540,22 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Exploración</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>el buhonero</t>
+          <t>56 escena(s) que no pasaron en 4 días</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>les falta: podía pasar (no tocó)</t>
         </is>
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>ej.: primera_gwin, primera_mirror, primera_armario, primera_stairs</t>
         </is>
       </c>
     </row>
@@ -31567,22 +31567,22 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Exploración</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Gertie Pye</t>
+          <t>38 escena(s) que no pasaron en 4 días</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>les falta: cuando se encuentran</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>ej.: diana_por_casualidad, par:ana+diana:0, par:ana+diana:1, par:ana+diana:2</t>
         </is>
       </c>
     </row>
@@ -31594,22 +31594,22 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Exploración</t>
         </is>
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Jane Andrews</t>
+          <t>19 escena(s) que no pasaron en 4 días</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>les falta: cuando Ana usa gwin</t>
         </is>
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>ej.: ventana_primavera_manana, ventana_primavera_tarde, ventana_verano_manana, ventana_verano_noche</t>
         </is>
       </c>
     </row>
@@ -31621,22 +31621,22 @@
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Exploración</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Prissy Andrews</t>
+          <t>13 escena(s) que no pasaron en 4 días</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>les falta: cuando Ana conversa con diana</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>ej.: conv_diana_pelo, conv_diana_minnie, conv_diana_nombres, conv_diana_escuela</t>
         </is>
       </c>
     </row>
@@ -31648,22 +31648,22 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Exploración</t>
         </is>
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Charlie Sloane</t>
+          <t>8 escena(s) que no pasaron en 4 días</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>les falta: ana no está en gg</t>
         </is>
       </c>
       <c r="E49" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>ej.: quiere_amiga, broche, prohibida, invita_allan</t>
         </is>
       </c>
     </row>
@@ -31675,22 +31675,22 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Exploración</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Moody Spurgeon</t>
+          <t>7 escena(s) que no pasaron en 4 días</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>les falta: cuando Ana conversa con marilla</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>ej.: conv_marilla_perdon, conv_marilla_cocina, conv_marilla_diana, conv_marilla_genio</t>
         </is>
       </c>
     </row>
@@ -31702,22 +31702,22 @@
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Exploración</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Tillie Boulter</t>
+          <t>6 escena(s) que no pasaron en 4 días</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>les falta: cuando Ana usa mirror</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>ej.: espejo_pelo, espejo_cordelia, espejo_tejas_verdes, espejo_zanahorias</t>
         </is>
       </c>
     </row>
@@ -31729,22 +31729,22 @@
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Exploración</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Felicity King</t>
+          <t>5 escena(s) que no pasaron en 4 días</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>les falta: cuando Ana conversa con matthew</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>ej.: conv_matthew_nombres, conv_matthew_mangas, conv_matthew_mujeres, conv_matthew_queens</t>
         </is>
       </c>
     </row>
@@ -31756,22 +31756,22 @@
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Exploración</t>
         </is>
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Felix King</t>
+          <t>4 escena(s) que no pasaron en 4 días</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>les falta: diana no está en Avonlea</t>
         </is>
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>ej.: conoce_diana, te_grosella, crup_aviso, cama_josephine</t>
         </is>
       </c>
     </row>
@@ -31783,22 +31783,22 @@
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Exploración</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Cecily King</t>
+          <t>4 escena(s) que no pasaron en 4 días</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>les falta: falta hecho:blewett_duda</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>ej.: duda_matthew, duda_suplica, duda_calla, devuelta_blewett</t>
         </is>
       </c>
     </row>
@@ -31810,22 +31810,22 @@
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Exploración</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Sara Stanley</t>
+          <t>4 escena(s) que no pasaron en 4 días</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>les falta: cuando Ana usa faro</t>
         </is>
       </c>
       <c r="E55" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>ej.: faro_verano, faro_invierno, faro_manana, faro_queens</t>
         </is>
       </c>
     </row>
@@ -31837,22 +31837,22 @@
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Noticias</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>el Sr. Phillips</t>
+          <t>«huerfano»: los Cuthbert van a traer un niño del orfanato</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>una escena o una frase con «sabe:quien:huerfano» (alguien que se entera y hace o dice algo)</t>
         </is>
       </c>
     </row>
@@ -31864,22 +31864,22 @@
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Noticias</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>el reverendo Allan</t>
+          <t>«cerdo_pye»: a los Pye se les escapó otra vez el cerdo</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>una escena o una frase con «sabe:quien:cerdo_pye» (alguien que se entera y hace o dice algo)</t>
         </is>
       </c>
     </row>
@@ -31891,22 +31891,22 @@
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Noticias</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>el Sr. Lawson</t>
+          <t>«maestra_plumas»: la maestra nueva usa sombrero con plumas</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>una escena o una frase con «sabe:quien:maestra_plumas» (alguien que se entera y hace o dice algo)</t>
         </is>
       </c>
     </row>
@@ -31918,22 +31918,22 @@
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Noticias</t>
         </is>
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>el herrero</t>
+          <t>«loro_harrison»: el loro del Sr. Harrison dice cosas terribles</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
         </is>
       </c>
       <c r="E59" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>una escena o una frase con «sabe:quien:loro_harrison» (alguien que se entera y hace o dice algo)</t>
         </is>
       </c>
     </row>
@@ -31945,22 +31945,22 @@
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Noticias</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>el editor de La Crónica</t>
+          <t>«rastrillo_matthew»: Matthew Cuthbert compró un rastrillo en invierno</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>una escena o una frase con «sabe:quien:rastrillo_matthew» (alguien que se entera y hace o dice algo)</t>
         </is>
       </c>
     </row>
@@ -31972,22 +31972,22 @@
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Noticias</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>la Srta. Hetty King</t>
+          <t>«ana_lengua»</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>es de Ana y no tiene versión exagerada</t>
         </is>
       </c>
       <c r="E61" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>una línea «exagerada:» (los chismosos la agrandan)</t>
         </is>
       </c>
     </row>
@@ -31999,22 +31999,22 @@
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Noticias</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Olivia King</t>
+          <t>«pastor_nuevo»: llegó un pastor nuevo, el Sr. Allan, con su esposa</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>una escena o una frase con «sabe:quien:pastor_nuevo» (alguien que se entera y hace o dice algo)</t>
         </is>
       </c>
     </row>
@@ -32026,22 +32026,22 @@
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Noticias</t>
         </is>
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>Jasper Dale</t>
+          <t>«tia_josephine»: la tía Josephine de los Barry vino de Charlottetown</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
         </is>
       </c>
       <c r="E63" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>una escena o una frase con «sabe:quien:tia_josephine» (alguien que se entera y hace o dice algo)</t>
         </is>
       </c>
     </row>
@@ -32053,22 +32053,22 @@
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Noticias</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Alec King</t>
+          <t>«se_va_phillips»: el Sr. Phillips se va de la escuela de Avonlea</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>nadie reacciona a ella (solo se cuenta); es un chisme del pueblo: puede bastar</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>una escena o una frase con «sabe:quien:se_va_phillips» (alguien que se entera y hace o dice algo)</t>
         </is>
       </c>
     </row>
@@ -32080,22 +32080,22 @@
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Llegadas</t>
         </is>
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Janet King</t>
+          <t>Prissy Andrews se va</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>nadie lo nota</t>
         </is>
       </c>
       <c r="E65" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>una noticia o una escena con «hecho:se_fue_prissy»</t>
         </is>
       </c>
     </row>
@@ -32107,22 +32107,22 @@
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Llegadas</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>la Sra. Pye</t>
+          <t>el buhonero llega (de visita)</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>tiene 2 frase(s) suelta(s)</t>
+          <t>nadie lo nota (solo queda en el diario)</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>una noticia «saben si hecho:llego_buhonero: …» o una escena «si: hecho:llego_buhonero»</t>
         </is>
       </c>
     </row>
@@ -32134,22 +32134,22 @@
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>Personas</t>
+          <t>Llegadas</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>el Sr. Sloane</t>
+          <t>una veraneante del hotel llega (de visita)</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr">
         <is>
-          <t>tiene 1 frase(s) suelta(s)</t>
+          <t>nadie lo nota (solo queda en el diario)</t>
         </is>
       </c>
       <c r="E67" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>una noticia «saben si hecho:llego_veraneante: …» o una escena «si: hecho:llego_veraneante»</t>
         </is>
       </c>
     </row>
@@ -32166,17 +32166,17 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>el Sr. Andrews</t>
+          <t>Presentación propia (cómo se presenta la primera vez)</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>tiene 1 frase(s) suelta(s)</t>
+          <t>32 usan la de siempre: Diana, el Sr. Shearer, el buhonero, el Sr. Phillips, el reverendo Allan, la Sra. Allan, el Sr. Lawson, el herrero, el editor de La Crónica, la Srta. Hetty King, Olivia King, Jasper Dale, Alec King, Janet King…</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>unas frases más en la hoja «Frases»</t>
+          <t>«presentacion» en personajes.json, o «presenta» en src/js/56-gente-de-avonlea.js, con su voz</t>
         </is>
       </c>
     </row>
@@ -32193,7 +32193,7 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Peg Bowen</t>
+          <t>el buhonero</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
@@ -32220,7 +32220,7 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>el Sr. Barry</t>
+          <t>Gertie Pye</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr">
@@ -32247,7 +32247,7 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Mary Joe</t>
+          <t>Jane Andrews</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
@@ -32274,7 +32274,7 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Jerry Buote</t>
+          <t>Prissy Andrews</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr">
@@ -32301,7 +32301,7 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>el médico</t>
+          <t>Charlie Sloane</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr">
@@ -32328,7 +32328,7 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>el Sr. Bell</t>
+          <t>Moody Spurgeon</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
@@ -32355,7 +32355,7 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>la Sra. Spencer</t>
+          <t>Tillie Boulter</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
@@ -32382,7 +32382,7 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>la Sra. Blewett</t>
+          <t>Felicity King</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr">
@@ -32409,7 +32409,7 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Carrie Sloane</t>
+          <t>Felix King</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr">
@@ -32436,7 +32436,7 @@
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>el jefe de estación</t>
+          <t>Cecily King</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr">
@@ -32463,12 +32463,12 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Thomas Lynde</t>
+          <t>Sara Stanley</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr">
         <is>
-          <t>tiene 1 frase(s) suelta(s)</t>
+          <t>tiene 2 frase(s) suelta(s)</t>
         </is>
       </c>
       <c r="E79" s="11" t="inlineStr">
@@ -32490,7 +32490,7 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>una veraneante del hotel</t>
+          <t>el Sr. Phillips</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr">
@@ -32517,12 +32517,12 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>un pescador</t>
+          <t>el reverendo Allan</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
         <is>
-          <t>tiene 1 frase(s) suelta(s)</t>
+          <t>tiene 2 frase(s) suelta(s)</t>
         </is>
       </c>
       <c r="E81" s="11" t="inlineStr">
@@ -32544,17 +32544,17 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Sin ninguna escena</t>
+          <t>el Sr. Lawson</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>42 de la gente del pueblo solo tienen frases sueltas: el buhonero, Josie Pye, Gertie Pye, Ruby Gillis, Jane Andrews, Prissy Andrews, Charlie Sloane, Moody Spurgeon, Tillie Boulter, Felicity King, Felix King, Cecily King, Sara Stanley, el Sr. Phillips, el reverendo Allan, el Sr. Lawson…</t>
+          <t>tiene 2 frase(s) suelta(s)</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>una escena pequeña para los que importan en el libro</t>
+          <t>unas frases más en la hoja «Frases»</t>
         </is>
       </c>
     </row>
@@ -32566,22 +32566,22 @@
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>Hechos</t>
+          <t>Personas</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>«ana_admite_gilbert»</t>
+          <t>el herrero</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr">
         <is>
-          <t>se deja y nadie lo lee: algo pasó y no tiene consecuencias</t>
+          <t>tiene 2 frase(s) suelta(s)</t>
         </is>
       </c>
       <c r="E83" s="11" t="inlineStr">
         <is>
-          <t>una escena, una frase o una noticia que lo recuerde</t>
+          <t>unas frases más en la hoja «Frases»</t>
         </is>
       </c>
     </row>
@@ -32593,22 +32593,22 @@
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>Hechos</t>
+          <t>Personas</t>
         </is>
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>«blewett_orgullo»</t>
+          <t>el editor de La Crónica</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>se deja y nadie lo lee: algo pasó y no tiene consecuencias</t>
+          <t>tiene 2 frase(s) suelta(s)</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>una escena, una frase o una noticia que lo recuerde</t>
+          <t>unas frases más en la hoja «Frases»</t>
         </is>
       </c>
     </row>
@@ -32620,22 +32620,22 @@
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>Hechos</t>
+          <t>Personas</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>«devuelta»</t>
+          <t>la Srta. Hetty King</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
         <is>
-          <t>se deja y nadie lo lee: algo pasó y no tiene consecuencias</t>
+          <t>tiene 2 frase(s) suelta(s)</t>
         </is>
       </c>
       <c r="E85" s="11" t="inlineStr">
         <is>
-          <t>una escena, una frase o una noticia que lo recuerde</t>
+          <t>unas frases más en la hoja «Frases»</t>
         </is>
       </c>
     </row>
@@ -32647,22 +32647,22 @@
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t>Hechos</t>
+          <t>Personas</t>
         </is>
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>«marilla_doblo_ropa»</t>
+          <t>Olivia King</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>se deja y nadie lo lee: algo pasó y no tiene consecuencias</t>
+          <t>tiene 2 frase(s) suelta(s)</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
         <is>
-          <t>una escena, una frase o una noticia que lo recuerde</t>
+          <t>unas frases más en la hoja «Frases»</t>
         </is>
       </c>
     </row>
@@ -32674,28 +32674,676 @@
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C87" s="11" t="inlineStr">
+        <is>
+          <t>Jasper Dale</t>
+        </is>
+      </c>
+      <c r="D87" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E87" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C88" s="11" t="inlineStr">
+        <is>
+          <t>Alec King</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E88" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C89" s="11" t="inlineStr">
+        <is>
+          <t>Janet King</t>
+        </is>
+      </c>
+      <c r="D89" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E89" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C90" s="11" t="inlineStr">
+        <is>
+          <t>la Sra. Pye</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E90" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B91" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C91" s="11" t="inlineStr">
+        <is>
+          <t>el Sr. Sloane</t>
+        </is>
+      </c>
+      <c r="D91" s="11" t="inlineStr">
+        <is>
+          <t>tiene 1 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E91" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B92" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C92" s="11" t="inlineStr">
+        <is>
+          <t>el Sr. Andrews</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="inlineStr">
+        <is>
+          <t>tiene 1 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E92" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C93" s="11" t="inlineStr">
+        <is>
+          <t>Peg Bowen</t>
+        </is>
+      </c>
+      <c r="D93" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E93" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C94" s="11" t="inlineStr">
+        <is>
+          <t>el Sr. Barry</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E94" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C95" s="11" t="inlineStr">
+        <is>
+          <t>Mary Joe</t>
+        </is>
+      </c>
+      <c r="D95" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E95" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C96" s="11" t="inlineStr">
+        <is>
+          <t>Jerry Buote</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E96" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C97" s="11" t="inlineStr">
+        <is>
+          <t>el médico</t>
+        </is>
+      </c>
+      <c r="D97" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E97" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C98" s="11" t="inlineStr">
+        <is>
+          <t>el Sr. Bell</t>
+        </is>
+      </c>
+      <c r="D98" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E98" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C99" s="11" t="inlineStr">
+        <is>
+          <t>la Sra. Spencer</t>
+        </is>
+      </c>
+      <c r="D99" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E99" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B100" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C100" s="11" t="inlineStr">
+        <is>
+          <t>la Sra. Blewett</t>
+        </is>
+      </c>
+      <c r="D100" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E100" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B101" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C101" s="11" t="inlineStr">
+        <is>
+          <t>Carrie Sloane</t>
+        </is>
+      </c>
+      <c r="D101" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E101" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B102" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C102" s="11" t="inlineStr">
+        <is>
+          <t>el jefe de estación</t>
+        </is>
+      </c>
+      <c r="D102" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E102" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C103" s="11" t="inlineStr">
+        <is>
+          <t>Thomas Lynde</t>
+        </is>
+      </c>
+      <c r="D103" s="11" t="inlineStr">
+        <is>
+          <t>tiene 1 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E103" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B104" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C104" s="11" t="inlineStr">
+        <is>
+          <t>una veraneante del hotel</t>
+        </is>
+      </c>
+      <c r="D104" s="11" t="inlineStr">
+        <is>
+          <t>tiene 2 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E104" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C105" s="11" t="inlineStr">
+        <is>
+          <t>un pescador</t>
+        </is>
+      </c>
+      <c r="D105" s="11" t="inlineStr">
+        <is>
+          <t>tiene 1 frase(s) suelta(s)</t>
+        </is>
+      </c>
+      <c r="E105" s="11" t="inlineStr">
+        <is>
+          <t>unas frases más en la hoja «Frases»</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B106" s="8" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="C106" s="11" t="inlineStr">
+        <is>
+          <t>Sin ninguna escena</t>
+        </is>
+      </c>
+      <c r="D106" s="11" t="inlineStr">
+        <is>
+          <t>42 de la gente del pueblo solo tienen frases sueltas: el buhonero, Josie Pye, Gertie Pye, Ruby Gillis, Jane Andrews, Prissy Andrews, Charlie Sloane, Moody Spurgeon, Tillie Boulter, Felicity King, Felix King, Cecily King, Sara Stanley, el Sr. Phillips, el reverendo Allan, el Sr. Lawson…</t>
+        </is>
+      </c>
+      <c r="E106" s="11" t="inlineStr">
+        <is>
+          <t>una escena pequeña para los que importan en el libro</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B107" s="8" t="inlineStr">
+        <is>
           <t>Hechos</t>
         </is>
       </c>
-      <c r="C87" s="11" t="inlineStr">
+      <c r="C107" s="11" t="inlineStr">
+        <is>
+          <t>«ana_admite_gilbert»</t>
+        </is>
+      </c>
+      <c r="D107" s="11" t="inlineStr">
+        <is>
+          <t>se deja y nadie lo lee: algo pasó y no tiene consecuencias</t>
+        </is>
+      </c>
+      <c r="E107" s="11" t="inlineStr">
+        <is>
+          <t>una escena, una frase o una noticia que lo recuerde</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B108" s="8" t="inlineStr">
+        <is>
+          <t>Hechos</t>
+        </is>
+      </c>
+      <c r="C108" s="11" t="inlineStr">
+        <is>
+          <t>«blewett_orgullo»</t>
+        </is>
+      </c>
+      <c r="D108" s="11" t="inlineStr">
+        <is>
+          <t>se deja y nadie lo lee: algo pasó y no tiene consecuencias</t>
+        </is>
+      </c>
+      <c r="E108" s="11" t="inlineStr">
+        <is>
+          <t>una escena, una frase o una noticia que lo recuerde</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B109" s="8" t="inlineStr">
+        <is>
+          <t>Hechos</t>
+        </is>
+      </c>
+      <c r="C109" s="11" t="inlineStr">
+        <is>
+          <t>«devuelta»</t>
+        </is>
+      </c>
+      <c r="D109" s="11" t="inlineStr">
+        <is>
+          <t>se deja y nadie lo lee: algo pasó y no tiene consecuencias</t>
+        </is>
+      </c>
+      <c r="E109" s="11" t="inlineStr">
+        <is>
+          <t>una escena, una frase o una noticia que lo recuerde</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>Hechos</t>
+        </is>
+      </c>
+      <c r="C110" s="11" t="inlineStr">
+        <is>
+          <t>«marilla_doblo_ropa»</t>
+        </is>
+      </c>
+      <c r="D110" s="11" t="inlineStr">
+        <is>
+          <t>se deja y nadie lo lee: algo pasó y no tiene consecuencias</t>
+        </is>
+      </c>
+      <c r="E110" s="11" t="inlineStr">
+        <is>
+          <t>una escena, una frase o una noticia que lo recuerde</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="8" t="inlineStr">
+        <is>
+          <t>baja</t>
+        </is>
+      </c>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>Hechos</t>
+        </is>
+      </c>
+      <c r="C111" s="11" t="inlineStr">
         <is>
           <t>«queens_primera»</t>
         </is>
       </c>
-      <c r="D87" s="11" t="inlineStr">
+      <c r="D111" s="11" t="inlineStr">
         <is>
           <t>se deja y nadie lo lee: algo pasó y no tiene consecuencias</t>
         </is>
       </c>
-      <c r="E87" s="11" t="inlineStr">
+      <c r="E111" s="11" t="inlineStr">
         <is>
           <t>una escena, una frase o una noticia que lo recuerde</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E87"/>
-  <conditionalFormatting sqref="A2:A87">
+  <autoFilter ref="A1:E111"/>
+  <conditionalFormatting sqref="A2:A111">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>A2="alta"</formula>
     </cfRule>

</xml_diff>

<commit_message>
El modelo de las interacciones: huecos e incoherencias con un solucionador lógico (Z3)
tools/modelo.py saca de los datos lo que cada uno le puede decir a Ana y el espacio de
situaciones posibles (día, hora, dónde está cada uno, cómo anda Ana, quién está en Avonlea,
qué pasó, a quién conoce), y pregunta por cada regla de src/datos/reglas.txt (lo único escrito
a mano: expectativas, imposibles, referencias) si existe una situación en que no se cumple.
Deja trazas/modelo.md y la hoja «Modelo» de la planilla. docs/MODELO_INTERACCIONES.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VY3w9XmL1TrbHxLtQe81Lv
</commit_message>
<xml_diff>
--- a/planilla/avonlea.xlsx
+++ b/planilla/avonlea.xlsx
@@ -9,26 +9,28 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cómo usar" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frases" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huecos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenas" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Noticias" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Llegadas" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diálogos" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hechos" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metas" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modelo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huecos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personas" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenas" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Noticias" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Llegadas" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diálogos" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hechos" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metas" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Frases'!$A$1:$J$2000</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cobertura'!$A$1:$E$111</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Personas'!$A$1:$H$55</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Escenas'!$A$1:$Q$164</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Noticias'!$A$1:$K$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Llegadas'!$A$1:$F$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Diálogos'!$A$1:$C$621</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Hechos'!$A$1:$D$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Modelo'!$A$1:$F$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cobertura'!$A$1:$E$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Personas'!$A$1:$H$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Escenas'!$A$1:$Q$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Noticias'!$A$1:$K$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Llegadas'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Diálogos'!$A$1:$C$621</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Hechos'!$A$1:$D$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,7 +592,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generada el 2026-10-16 07:00 desde los datos del juego (node tools/planilla.js).</t>
+          <t>Generada el 2026-10-16 07:20 desde los datos del juego (node tools/planilla.js).</t>
         </is>
       </c>
     </row>
@@ -773,6 +775,272 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Quién</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>De visita</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Llega si… (una alternativa por línea)</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Se va si… (una por línea)</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Al llegar (diario)</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Al irse (diario)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>diana</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="n"/>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>dias_desde:llegada_tv:17</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="n"/>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>Diana Barry volvió de Carmody, donde su tía.</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>gilbert</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n"/>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>dias_desde:escuela:4
+estacion:invierno</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="n"/>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Gilbert Blythe volvió de Nuevo Brunswick.</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>josephine</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>estacion:invierno</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>La tía Josephine llegó de Charlottetown a La Cuesta del Huerto.</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>La tía Josephine se volvió a Charlottetown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>allan</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n"/>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>estacion:primavera, dias_desde:se_fue_josephine:7</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Llegó el pastor nuevo, el Sr. Allan, con su esposa.</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>sraallan</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n"/>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>estacion:primavera, dias_desde:se_fue_josephine:7</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>phillips</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>estacion:verano, hecho:llego_josephine</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>El Sr. Phillips se despidió de la escuela: todas las niñas lloraron.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>prissy</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>hecho:se_fue_phillips</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Prissy Andrews se fue a Queen's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>stacy</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>estacion:otoño, hecho:se_fue_phillips</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Llegó la maestra nueva, la Srta. Stacy.</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>buhonero</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>dia_estacion:4
+dia_estacion:11</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>veraneante</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>estacion:verano</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F11"/>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B211" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"sí"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11350,7 +11618,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12982,7 +13250,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -30334,6 +30602,3618 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F119"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Regla</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Quién</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Tiene</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Una situación</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Lo que falta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>algo que decirle</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Gertie Pye</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>día: 71 · estación: verano · hora: 6:00 · Ana en: el patio de Tejas Verdes · conoce a Gertie Pye: sí</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>dias_desde:escuela:3 (2); !conoce:gertie (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Alec King</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a Alec King: sí</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>el reverendo Allan</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a el reverendo Allan: sí</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Andrews</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a el Sr. Andrews: sí</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Barry</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a la Sra. Barry: no</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>hora:7-21 (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Blewett</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a la Sra. Blewett: sí</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>el buhonero</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a el buhonero: sí</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>el editor de La Crónica</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a el editor de La Crónica: sí</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>el capitán Jim</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: La Cuesta del Huerto · Ana: en camisón · conoce a el capitán Jim: sí</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Harrison</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a el Sr. Harrison: sí</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>el herrero</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: La Cuesta del Huerto · Ana: en camisón · conoce a el herrero: sí</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>la Srta. Hetty King</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a la Srta. Hetty King: sí</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Janet King</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a Janet King: sí</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Jasper Dale</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a Jasper Dale: sí</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>el jefe de estación</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a el jefe de estación: sí</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Jerry Buote</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a Jerry Buote: sí</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>la Srta. Josephine Barry</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: La Cuesta del Huerto · Ana: en camisón · conoce a la Srta. Josephine Barry: no</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Lawson</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a el Sr. Lawson: sí</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Lynde</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a la Sra. Lynde: no</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>hora:7-21 (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Marilla</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a Marilla: sí</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>hora:9-19 (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Mary Joe</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: la casa del Sr. Harrison · Ana: en camisón · conoce a Mary Joe: sí</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Matthew</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a Matthew: sí</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>el médico</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a el médico: sí</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Olivia King</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a Olivia King: sí</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Peg Bowen</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a Peg Bowen: sí</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>un pescador</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>día: 71 · estación: verano · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a un pescador: sí</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Phillips</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a el Sr. Phillips: sí</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Shearer</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a el Sr. Shearer: sí</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Sloane</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a el Sr. Sloane: sí</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Spencer</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a la Sra. Spencer: sí</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Allan</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: La Cuesta del Huerto · Ana: en camisón · conoce a la Sra. Allan: sí</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Pye</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a la Sra. Pye: sí</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Barry</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: La Cuesta del Huerto · Ana: en camisón · conoce a el Sr. Barry: sí</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Bell</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: la tienda de Lawson · Ana: en camisón · conoce a el Sr. Bell: sí</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>la Srta. Stacy</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 6:00 · Ana en: el camino o la aldea · Ana: en camisón · conoce a la Srta. Stacy: sí</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Thomas Lynde</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: la casa de la Sra. Lynde · Ana: en camisón · conoce a Thomas Lynde: sí</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>un vecino (sin nombre)</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 6:00 · Ana en: la iglesia · Ana: en camisón · conoce a un vecino (sin nombre): no</t>
+        </is>
+      </c>
+      <c r="F38" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>reacciona al camisón fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>una veraneante del hotel</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>día: 71 · estación: verano · hora: 6:00 · Ana en: La Cuesta del Huerto · Ana: en camisón · conoce a una veraneante del hotel: sí</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Alec King</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>día: 67 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a Alec King: sí</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>el reverendo Allan</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>día: 113 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el reverendo Allan: sí</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Andrews</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>día: 71 · estación: verano · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el Sr. Andrews: sí</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Barry</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a la Sra. Barry: no</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Blewett</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>día: 1 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a la Sra. Blewett: sí</t>
+        </is>
+      </c>
+      <c r="F44" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>el buhonero</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>día: 11 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el buhonero: sí</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>el editor de La Crónica</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el editor de La Crónica: sí</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>el capitán Jim</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>día: 126 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el capitán Jim: sí</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Harrison</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>día: 3 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el Sr. Harrison: sí</t>
+        </is>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>el herrero</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el herrero: sí</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>la Srta. Hetty King</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a la Srta. Hetty King: sí</t>
+        </is>
+      </c>
+      <c r="F50" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Janet King</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a Janet King: sí</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>Jasper Dale</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a Jasper Dale: sí</t>
+        </is>
+      </c>
+      <c r="F52" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>el jefe de estación</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="11" t="inlineStr">
+        <is>
+          <t>día: 71 · estación: verano · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el jefe de estación: sí</t>
+        </is>
+      </c>
+      <c r="F53" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>Jerry Buote</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>día: 1 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a Jerry Buote: sí</t>
+        </is>
+      </c>
+      <c r="F54" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>la Srta. Josephine Barry</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a la Srta. Josephine Barry: no</t>
+        </is>
+      </c>
+      <c r="F55" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Lawson</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el Sr. Lawson: sí</t>
+        </is>
+      </c>
+      <c r="F56" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Lynde</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a la Sra. Lynde: no</t>
+        </is>
+      </c>
+      <c r="F57" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Marilla</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a Marilla: sí</t>
+        </is>
+      </c>
+      <c r="F58" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>Mary Joe</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a Mary Joe: sí</t>
+        </is>
+      </c>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>Matthew</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a Matthew: sí</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>el médico</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" s="11" t="inlineStr">
+        <is>
+          <t>día: 85 · estación: otoño · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el médico: sí</t>
+        </is>
+      </c>
+      <c r="F61" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>Olivia King</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" s="11" t="inlineStr">
+        <is>
+          <t>día: 1 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a Olivia King: sí</t>
+        </is>
+      </c>
+      <c r="F62" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>Peg Bowen</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a Peg Bowen: sí</t>
+        </is>
+      </c>
+      <c r="F63" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>un pescador</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a un pescador: sí</t>
+        </is>
+      </c>
+      <c r="F64" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Phillips</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el Sr. Phillips: sí</t>
+        </is>
+      </c>
+      <c r="F65" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Shearer</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el Sr. Shearer: sí</t>
+        </is>
+      </c>
+      <c r="F66" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B67" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Sloane</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el Sr. Sloane: sí</t>
+        </is>
+      </c>
+      <c r="F67" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Spencer</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a la Sra. Spencer: sí</t>
+        </is>
+      </c>
+      <c r="F68" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Allan</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a la Sra. Allan: sí</t>
+        </is>
+      </c>
+      <c r="F69" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Pye</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a la Sra. Pye: sí</t>
+        </is>
+      </c>
+      <c r="F70" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Barry</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el Sr. Barry: sí</t>
+        </is>
+      </c>
+      <c r="F71" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Bell</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a el Sr. Bell: sí</t>
+        </is>
+      </c>
+      <c r="F72" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>la Srta. Stacy</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="11" t="inlineStr">
+        <is>
+          <t>día: 113 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a la Srta. Stacy: sí</t>
+        </is>
+      </c>
+      <c r="F73" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>Thomas Lynde</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a Thomas Lynde: sí</t>
+        </is>
+      </c>
+      <c r="F74" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>un vecino (sin nombre)</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="11" t="inlineStr">
+        <is>
+          <t>día: 113 · estación: primavera · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a un vecino (sin nombre): no</t>
+        </is>
+      </c>
+      <c r="F75" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana está sin sombrero en la iglesia</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>una veraneante del hotel</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="11" t="inlineStr">
+        <is>
+          <t>día: 127 · estación: verano · hora: 6:00 · Ana en: la iglesia · Ana: sin sombrero · conoce a una veraneante del hotel: sí</t>
+        </is>
+      </c>
+      <c r="F76" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>Alec King</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a Alec King: sí</t>
+        </is>
+      </c>
+      <c r="F77" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>el reverendo Allan</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el reverendo Allan: sí</t>
+        </is>
+      </c>
+      <c r="F78" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Andrews</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el Sr. Andrews: sí</t>
+        </is>
+      </c>
+      <c r="F79" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Barry</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 21:00 · Ana en: el camino o la aldea · conoce a la Sra. Barry: no</t>
+        </is>
+      </c>
+      <c r="F80" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Blewett</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a la Sra. Blewett: sí</t>
+        </is>
+      </c>
+      <c r="F81" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>el buhonero</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" s="11" t="inlineStr">
+        <is>
+          <t>día: 102 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el buhonero: sí</t>
+        </is>
+      </c>
+      <c r="F82" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>el editor de La Crónica</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 21:00 · Ana en: el camino o la aldea · conoce a el editor de La Crónica: sí</t>
+        </is>
+      </c>
+      <c r="F83" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>el capitán Jim</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el capitán Jim: sí</t>
+        </is>
+      </c>
+      <c r="F84" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Harrison</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el Sr. Harrison: sí</t>
+        </is>
+      </c>
+      <c r="F85" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>el herrero</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el herrero: sí</t>
+        </is>
+      </c>
+      <c r="F86" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>la Srta. Hetty King</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a la Srta. Hetty King: sí</t>
+        </is>
+      </c>
+      <c r="F87" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>Janet King</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a Janet King: sí</t>
+        </is>
+      </c>
+      <c r="F88" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>Jasper Dale</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a Jasper Dale: sí</t>
+        </is>
+      </c>
+      <c r="F89" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>el jefe de estación</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el jefe de estación: sí</t>
+        </is>
+      </c>
+      <c r="F90" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B91" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>Jerry Buote</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" s="11" t="inlineStr">
+        <is>
+          <t>día: 1 · estación: primavera · hora: 21:00 · Ana en: el camino o la aldea · conoce a Jerry Buote: sí</t>
+        </is>
+      </c>
+      <c r="F91" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B92" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>la Srta. Josephine Barry</t>
+        </is>
+      </c>
+      <c r="D92" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a la Srta. Josephine Barry: no</t>
+        </is>
+      </c>
+      <c r="F92" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Lawson</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el Sr. Lawson: sí</t>
+        </is>
+      </c>
+      <c r="F93" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Lynde</t>
+        </is>
+      </c>
+      <c r="D94" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a la Sra. Lynde: no</t>
+        </is>
+      </c>
+      <c r="F94" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>Marilla</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a Marilla: sí</t>
+        </is>
+      </c>
+      <c r="F95" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>Mary Joe</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 21:00 · Ana en: La Cuesta del Huerto · conoce a Mary Joe: sí</t>
+        </is>
+      </c>
+      <c r="F96" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>Matthew</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a Matthew: sí</t>
+        </is>
+      </c>
+      <c r="F97" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>el médico</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el médico: sí</t>
+        </is>
+      </c>
+      <c r="F98" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>Olivia King</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a Olivia King: sí</t>
+        </is>
+      </c>
+      <c r="F99" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B100" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>Peg Bowen</t>
+        </is>
+      </c>
+      <c r="D100" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a Peg Bowen: sí</t>
+        </is>
+      </c>
+      <c r="F100" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B101" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>un pescador</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a un pescador: sí</t>
+        </is>
+      </c>
+      <c r="F101" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B102" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Phillips</t>
+        </is>
+      </c>
+      <c r="D102" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el Sr. Phillips: sí</t>
+        </is>
+      </c>
+      <c r="F102" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Shearer</t>
+        </is>
+      </c>
+      <c r="D103" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E103" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el Sr. Shearer: sí</t>
+        </is>
+      </c>
+      <c r="F103" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B104" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Sloane</t>
+        </is>
+      </c>
+      <c r="D104" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E104" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el Sr. Sloane: sí</t>
+        </is>
+      </c>
+      <c r="F104" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Spencer</t>
+        </is>
+      </c>
+      <c r="D105" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a la Sra. Spencer: sí</t>
+        </is>
+      </c>
+      <c r="F105" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B106" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Allan</t>
+        </is>
+      </c>
+      <c r="D106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 21:00 · Ana en: el camino o la aldea · conoce a la Sra. Allan: sí</t>
+        </is>
+      </c>
+      <c r="F106" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B107" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Pye</t>
+        </is>
+      </c>
+      <c r="D107" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a la Sra. Pye: sí</t>
+        </is>
+      </c>
+      <c r="F107" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B108" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Barry</t>
+        </is>
+      </c>
+      <c r="D108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 21:00 · Ana en: el camino o la aldea · conoce a el Sr. Barry: sí</t>
+        </is>
+      </c>
+      <c r="F108" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B109" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Bell</t>
+        </is>
+      </c>
+      <c r="D109" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a el Sr. Bell: sí</t>
+        </is>
+      </c>
+      <c r="F109" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>la Srta. Stacy</t>
+        </is>
+      </c>
+      <c r="D110" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 21:00 · Ana en: el camino o la aldea · conoce a la Srta. Stacy: sí</t>
+        </is>
+      </c>
+      <c r="F110" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>Thomas Lynde</t>
+        </is>
+      </c>
+      <c r="D111" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a Thomas Lynde: sí</t>
+        </is>
+      </c>
+      <c r="F111" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t>un vecino (sin nombre)</t>
+        </is>
+      </c>
+      <c r="D112" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E112" s="11" t="inlineStr">
+        <is>
+          <t>día: 46 · estación: invierno · hora: 21:00 · Ana en: el camino o la aldea · conoce a un vecino (sin nombre): no</t>
+        </is>
+      </c>
+      <c r="F112" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="8" t="inlineStr">
+        <is>
+          <t>hueco</t>
+        </is>
+      </c>
+      <c r="B113" s="8" t="inlineStr">
+        <is>
+          <t>reacciona si Ana anda sola de noche</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>una veraneante del hotel</t>
+        </is>
+      </c>
+      <c r="D113" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E113" s="11" t="inlineStr">
+        <is>
+          <t>día: 71 · estación: verano · hora: 21:00 · Ana en: el camino o la aldea · conoce a una veraneante del hotel: sí</t>
+        </is>
+      </c>
+      <c r="F113" s="11" t="inlineStr">
+        <is>
+          <t>no tiene ninguna</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="8" t="inlineStr">
+        <is>
+          <t>incoherencia</t>
+        </is>
+      </c>
+      <c r="B114" s="8" t="inlineStr">
+        <is>
+          <t>«pasa» invita a entrar</t>
+        </is>
+      </c>
+      <c r="C114" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Barry</t>
+        </is>
+      </c>
+      <c r="D114" s="8" t="inlineStr">
+        <is>
+          <t>frase de invierno</t>
+        </is>
+      </c>
+      <c r="E114" s="11" t="inlineStr">
+        <is>
+          <t>día: 99 · estación: invierno · hora: 6:00 · Ana en: la casa de la Sra. Lynde · conoce a la Sra. Barry: sí</t>
+        </is>
+      </c>
+      <c r="F114" s="11" t="inlineStr">
+        <is>
+          <t>«Pasa, pasa, que hace un frío terrible. Diana está junto al fuego.» exige donde:barry:propia</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="8" t="inlineStr">
+        <is>
+          <t>incoherencia</t>
+        </is>
+      </c>
+      <c r="B115" s="8" t="inlineStr">
+        <is>
+          <t>«pasa» invita a entrar</t>
+        </is>
+      </c>
+      <c r="C115" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Lynde</t>
+        </is>
+      </c>
+      <c r="D115" s="8" t="inlineStr">
+        <is>
+          <t>frase de invierno</t>
+        </is>
+      </c>
+      <c r="E115" s="11" t="inlineStr">
+        <is>
+          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: la cocina de Tejas Verdes · conoce a la Sra. Lynde: sí</t>
+        </is>
+      </c>
+      <c r="F115" s="11" t="inlineStr">
+        <is>
+          <t>«Pasa, niña, que hace un frío de mil demonios... perdón, de los que dan escalofrí» exige donde:lynde:propia</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="8" t="inlineStr">
+        <is>
+          <t>incoherencia</t>
+        </is>
+      </c>
+      <c r="B116" s="8" t="inlineStr">
+        <is>
+          <t>la Srta. Stacy, cuando ya llegó</t>
+        </is>
+      </c>
+      <c r="C116" s="8" t="inlineStr">
+        <is>
+          <t>Carrie Sloane</t>
+        </is>
+      </c>
+      <c r="D116" s="8" t="inlineStr">
+        <is>
+          <t>frase</t>
+        </is>
+      </c>
+      <c r="E116" s="11" t="inlineStr">
+        <is>
+          <t>día: 88 · estación: otoño · hora: 6:00 · Ana en: el camino o la aldea · conoce a Carrie Sloane: sí</t>
+        </is>
+      </c>
+      <c r="F116" s="11" t="inlineStr">
+        <is>
+          <t>«¿Viste la composición de Ana? ¡La señorita Stacy la leyó en voz alta!» exige hecho:llego_stacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="8" t="inlineStr">
+        <is>
+          <t>incoherencia</t>
+        </is>
+      </c>
+      <c r="B117" s="8" t="inlineStr">
+        <is>
+          <t>Gilbert, cuando ya volvió</t>
+        </is>
+      </c>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>Diana</t>
+        </is>
+      </c>
+      <c r="D117" s="8" t="inlineStr">
+        <is>
+          <t>escena al encontrarse</t>
+        </is>
+      </c>
+      <c r="E117" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: su pieza · conoce a Diana: sí</t>
+        </is>
+      </c>
+      <c r="F117" s="11" t="inlineStr">
+        <is>
+          <t>«diana: Gilbert Blythe te miró otra vez en clase.» exige hecho:llego_gilbert</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="8" t="inlineStr">
+        <is>
+          <t>incoherencia</t>
+        </is>
+      </c>
+      <c r="B118" s="8" t="inlineStr">
+        <is>
+          <t>«saludos a Marilla», fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>la Sra. Barry</t>
+        </is>
+      </c>
+      <c r="D118" s="8" t="inlineStr">
+        <is>
+          <t>frase</t>
+        </is>
+      </c>
+      <c r="E118" s="11" t="inlineStr">
+        <is>
+          <t>día: 60 · estación: primavera · hora: 6:00 · Ana en: la cocina de Tejas Verdes · conoce a la Sra. Barry: no</t>
+        </is>
+      </c>
+      <c r="F118" s="11" t="inlineStr">
+        <is>
+          <t>«Saluda a Marilla de mi parte.» exige !donde:ana:tejas</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="8" t="inlineStr">
+        <is>
+          <t>incoherencia</t>
+        </is>
+      </c>
+      <c r="B119" s="8" t="inlineStr">
+        <is>
+          <t>«saludos a Marilla», fuera de Tejas Verdes</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>un vecino (sin nombre)</t>
+        </is>
+      </c>
+      <c r="D119" s="8" t="inlineStr">
+        <is>
+          <t>frase</t>
+        </is>
+      </c>
+      <c r="E119" s="11" t="inlineStr">
+        <is>
+          <t>día: 57 · estación: primavera · hora: 6:00 · Ana en: el patio de Tejas Verdes · conoce a un vecino (sin nombre): no</t>
+        </is>
+      </c>
+      <c r="F119" s="11" t="inlineStr">
+        <is>
+          <t>«¡Qué grande estás, niña! Saludos a Marilla.» exige !donde:ana:tejas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F119"/>
+  <conditionalFormatting sqref="A2:A119">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>A2="incoherencia"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -33355,7 +37235,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -37113,7 +40993,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -38275,7 +42155,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40157,7 +44037,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -48595,7 +52475,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -49118,270 +52998,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Quién</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>De visita</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>Llega si… (una alternativa por línea)</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="inlineStr">
-        <is>
-          <t>Se va si… (una por línea)</t>
-        </is>
-      </c>
-      <c r="E1" s="6" t="inlineStr">
-        <is>
-          <t>Al llegar (diario)</t>
-        </is>
-      </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>Al irse (diario)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>diana</t>
-        </is>
-      </c>
-      <c r="B2" s="9" t="n"/>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
-          <t>dias_desde:llegada_tv:17</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="n"/>
-      <c r="E2" s="9" t="inlineStr">
-        <is>
-          <t>Diana Barry volvió de Carmody, donde su tía.</t>
-        </is>
-      </c>
-      <c r="F2" s="9" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>gilbert</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="n"/>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>dias_desde:escuela:4
-estacion:invierno</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="n"/>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>Gilbert Blythe volvió de Nuevo Brunswick.</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>josephine</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>estacion:invierno</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="n"/>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>La tía Josephine llegó de Charlottetown a La Cuesta del Huerto.</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>La tía Josephine se volvió a Charlottetown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>allan</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="n"/>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>estacion:primavera, dias_desde:se_fue_josephine:7</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="inlineStr">
-        <is>
-          <t>Llegó el pastor nuevo, el Sr. Allan, con su esposa.</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>sraallan</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="n"/>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>estacion:primavera, dias_desde:se_fue_josephine:7</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="9" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>phillips</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>estacion:verano, hecho:llego_josephine</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>El Sr. Phillips se despidió de la escuela: todas las niñas lloraron.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>prissy</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>hecho:se_fue_phillips</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>Prissy Andrews se fue a Queen's.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>stacy</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>estacion:otoño, hecho:se_fue_phillips</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Llegó la maestra nueva, la Srta. Stacy.</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>buhonero</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>dia_estacion:4
-dia_estacion:11</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>veraneante</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>estacion:verano</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="n"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F11"/>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B211" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"sí"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Partida 8 (test de usuaria): de cada error, una regla general
- Lo que se ve de Ana se dice desde donde se ve, aunque estén en misa, y antes que una conversación
- Prueba nueva tools/reacciones.js: el juego dice la reacción, sola (con el motor de antes, falla)
- Las noticias: «la callan» (lo que avergüenza a la casa no se cuenta afuera), «callados» (Thomas, Matthew),
  una frase que nombra a alguien no se le dice ni la dice esa persona
- grafo.js: una noticia que dice «anoche» u «hoy» no se cuenta por días
- El mapa: tocar el dibujo o el nombre de un lugar es ir a ese lugar
- docs/MODELO_INTERACCIONES.md: «De un error a una regla»; trazas/partida8

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VY3w9XmL1TrbHxLtQe81Lv
</commit_message>
<xml_diff>
--- a/planilla/avonlea.xlsx
+++ b/planilla/avonlea.xlsx
@@ -23,7 +23,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Frases'!$A$1:$J$2000</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Modelo'!$A$1:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Modelo'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cobertura'!$A$1:$E$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Personas'!$A$1:$H$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Escenas'!$A$1:$Q$166</definedName>
@@ -592,7 +592,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generada el 2026-10-16 13:43 desde los datos del juego (node tools/planilla.js).</t>
+          <t>Generada el 2026-10-16 14:19 desde los datos del juego (node tools/planilla.js).</t>
         </is>
       </c>
     </row>
@@ -31801,7 +31801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31844,173 +31844,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>incoherencia</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>«en camisón por el camino», cuando la ven fuera de Tejas Verdes</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>Marilla</t>
-        </is>
-      </c>
-      <c r="D2" s="8" t="inlineStr">
-        <is>
-          <t>escena</t>
-        </is>
-      </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: su pieza · conoce a Marilla: sí</t>
-        </is>
-      </c>
-      <c r="F2" s="11" t="inlineStr">
-        <is>
-          <t>«marilla: Ana. Me vino a contar alguien que andabas en camisón por Avonlea. En ca» exige !donde:ana:tejas</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>incoherencia</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>«en camisón por el camino», cuando la ven fuera de Tejas Verdes</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Marilla</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>escena</t>
-        </is>
-      </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>día: 43 · estación: invierno · hora: 6:00 · Ana en: su pieza · conoce a Marilla: sí</t>
-        </is>
-      </c>
-      <c r="F3" s="11" t="inlineStr">
-        <is>
-          <t>«marilla: Ana. Alguien me dijo que anoche te vieron sola por el camino, a esas ho» exige !donde:ana:tejas</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>incoherencia</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>«en camisón por el camino», cuando la ven fuera de Tejas Verdes</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>la Sra. Barry</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>escena</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>día: 57 · estación: primavera · hora: 7:00 · Ana en: el patio de Tejas Verdes · Ana: en camisón · conoce a la Sra. Barry: sí</t>
-        </is>
-      </c>
-      <c r="F4" s="11" t="inlineStr">
-        <is>
-          <t>«barry: (La Sra. Barry se lleva la mano al pecho.) ¡Niña! ¿Andas en camisón por l» exige !donde:ana:tejas</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>incoherencia</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>«en camisón por el camino», cuando la ven fuera de Tejas Verdes</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>la Sra. Lynde</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>escena</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>día: 46 · estación: invierno · hora: 7:00 · Ana en: la cocina de Tejas Verdes · Ana: en camisón · conoce a la Sra. Lynde: no</t>
-        </is>
-      </c>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>«lynde: ¡Habráse visto! ¡La huérfana de los Cuthbert, en camisón por el camino! E» exige !donde:ana:tejas</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>incoherencia</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>«en camisón por el camino», cuando la ven fuera de Tejas Verdes</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>la Srta. Hetty King</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>frase</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>día: 46 · estación: invierno · hora: 6:00 · Ana en: la cocina de Tejas Verdes · conoce a la Srta. Hetty King: sí</t>
-        </is>
-      </c>
-      <c r="F6" s="11" t="inlineStr">
-        <is>
-          <t>«Señorita, no se corre por la calle principal. ¡Y menos con el sombrero torcido!» exige !donde:ana:tejas</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F6"/>
-  <conditionalFormatting sqref="A2:A6">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>A2="incoherencia"</formula>
-    </cfRule>
-  </conditionalFormatting>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -51131,7 +50966,7 @@
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>¿Supo que anoche vieron a la niña de los Cuthbert sola por el camino? ¡A esas horas!</t>
+          <t>¿Supo que vieron a la niña de los Cuthbert sola por el camino, de noche? ¡A esas horas!</t>
         </is>
       </c>
       <c r="I15" s="9" t="n"/>

</xml_diff>

<commit_message>
Antes de que la acepten: nada supone que Ana se queda
- reglas.txt: lo que habla de su futuro en Avonlea (la escuela, la escuela dominical, «el año que viene») pide hecho:se_queda
- reglas.txt: nunca el día 5 sin se_queda (Marilla decide el día 3, o Ana se va y el juego termina)
- frases de Tillie, el Sr. Bell y el reverendo Allan: después de que se queda

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VY3w9XmL1TrbHxLtQe81Lv
</commit_message>
<xml_diff>
--- a/planilla/avonlea.xlsx
+++ b/planilla/avonlea.xlsx
@@ -23,7 +23,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Frases'!$A$1:$J$2000</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Modelo'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Modelo'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cobertura'!$A$1:$E$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Personas'!$A$1:$H$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Escenas'!$A$1:$Q$166</definedName>
@@ -592,7 +592,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generada el 2026-10-16 14:19 desde los datos del juego (node tools/planilla.js).</t>
+          <t>Generada el 2026-10-16 15:01 desde los datos del juego (node tools/planilla.js).</t>
         </is>
       </c>
     </row>
@@ -13488,7 +13488,7 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>escena lynde_visita, escena ventana_se_queda, escena espejo_tejas_verdes, escena armario_vestidos, escena lugar_camino_blanco_flor, escena lugar_primera_nieve, un comentario de espejo, una frase de matthew, una frase de marilla, una frase de lynde, meta conocer_diana</t>
+          <t>escena lynde_visita, escena ventana_se_queda, escena espejo_tejas_verdes, escena armario_vestidos, escena lugar_camino_blanco_flor, escena lugar_primera_nieve, un comentario de espejo, una frase de matthew, una frase de marilla, una frase de lynde, una frase de tillie, una frase de allan, una frase de srbell, meta conocer_diana</t>
         </is>
       </c>
       <c r="D96" s="8" t="inlineStr"/>
@@ -17986,7 +17986,11 @@
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr"/>
-      <c r="F114" s="7" t="inlineStr"/>
+      <c r="F114" s="7" t="inlineStr">
+        <is>
+          <t>se_queda</t>
+        </is>
+      </c>
       <c r="G114" s="7" t="n"/>
       <c r="H114" s="7" t="inlineStr"/>
       <c r="I114" s="7" t="inlineStr"/>
@@ -18404,7 +18408,11 @@
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr"/>
-      <c r="F128" s="7" t="inlineStr"/>
+      <c r="F128" s="7" t="inlineStr">
+        <is>
+          <t>se_queda</t>
+        </is>
+      </c>
       <c r="G128" s="7" t="n"/>
       <c r="H128" s="7" t="inlineStr"/>
       <c r="I128" s="7" t="inlineStr"/>
@@ -19924,7 +19932,11 @@
         </is>
       </c>
       <c r="E182" s="7" t="inlineStr"/>
-      <c r="F182" s="7" t="inlineStr"/>
+      <c r="F182" s="7" t="inlineStr">
+        <is>
+          <t>se_queda</t>
+        </is>
+      </c>
       <c r="G182" s="7" t="n"/>
       <c r="H182" s="7" t="inlineStr"/>
       <c r="I182" s="7" t="inlineStr"/>
@@ -31801,7 +31813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31844,8 +31856,109 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>incoherencia</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>lo que supone que Ana se queda, cuando ya se queda</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Tillie Boulter</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>frase</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>día: 1 · estación: primavera · hora: 6:00 · Ana en: el patio de Tejas Verdes · conoce a Tillie Boulter: sí</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>«Encontré un nido de petirrojos detrás de la escuela. ¡No le digas a nadie!» exige hecho:se_queda</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>incoherencia</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>lo que supone que Ana se queda, cuando ya se queda</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>el reverendo Allan</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>frase</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>día: 1 · estación: primavera · hora: 6:00 · Ana en: el patio de Tejas Verdes · conoce a el reverendo Allan: sí</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>«Que Dios te bendiga, Ana. ¿Te veremos el domingo en la escuela dominical?» exige hecho:se_queda</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>incoherencia</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>lo que supone que Ana se queda, cuando ya se queda</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>el Sr. Bell</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>frase</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>día: 1 · estación: primavera · hora: 6:00 · Ana en: la cocina de Tejas Verdes · conoce a el Sr. Bell: sí</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>«Te esperamos el domingo en la escuela dominical, Ana. Y apréndete el versículo.» exige hecho:se_queda</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:F4"/>
+  <conditionalFormatting sqref="A2:A4">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>A2="incoherencia"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -36064,10 +36177,10 @@
         </is>
       </c>
       <c r="C22" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22" s="19" t="n">
         <v>2</v>
@@ -37767,7 +37880,7 @@
         <v>1</v>
       </c>
       <c r="D49" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E49" s="19" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Los días a prueba: metas, reglas y guiños
- cuaderno.txt: solo rezar, ayudar, la huerta y los nombres se pueden hacer antes de que acepten a Ana («a prueba»);
  las demás piden «quedarse» (grafo.js lo revisa)
- reglas.txt: Marilla y Matthew, mientras está a prueba, tienen algo que lo tenga en cuenta; «ojalá te quedes» o
  «devolverte», solo mientras no se sabe
- los guiños del cuaderno: con [condiciones], como las frases; el modelo ahora los lee (encontró los de Diana
  mientras se lo prohíben)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VY3w9XmL1TrbHxLtQe81Lv
</commit_message>
<xml_diff>
--- a/planilla/avonlea.xlsx
+++ b/planilla/avonlea.xlsx
@@ -23,7 +23,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Frases'!$A$1:$J$2000</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Modelo'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Modelo'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cobertura'!$A$1:$E$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Personas'!$A$1:$H$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Escenas'!$A$1:$Q$166</definedName>
@@ -592,7 +592,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generada el 2026-10-16 15:01 desde los datos del juego (node tools/planilla.js).</t>
+          <t>Generada el 2026-10-16 17:36 desde los datos del juego (node tools/planilla.js).</t>
         </is>
       </c>
     </row>
@@ -13774,7 +13774,7 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>hecho:diana_borracha</t>
+          <t>quedarse, hecho:diana_borracha</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
@@ -13826,7 +13826,11 @@
           <t>Visitar a la Sra. Lynde</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr"/>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>quedarse</t>
+        </is>
+      </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
           <t>Vive en la Hondonada, junto al camino; desde su ventana lo ve todo. Por la tarde está en casa.</t>
@@ -13899,7 +13903,11 @@
           <t>Hacerle un regalo a Marilla que le guste</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr"/>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>quedarse</t>
+        </is>
+      </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
           <t>A Marilla le gusta lo hecho a mano. Las flores de la huerta también alegran.</t>
@@ -13968,7 +13976,11 @@
           <t>Ir a la escuela dominical</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr"/>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>quedarse</t>
+        </is>
+      </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
           <t>En la iglesia, camino a Bright River.</t>
@@ -13991,7 +14003,11 @@
           <t>Ir a la escuela</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr"/>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>quedarse</t>
+        </is>
+      </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
           <t>La escuela está junto al río, más allá de la aldea. Allí van Diana, Gilbert Blythe y los demás.</t>
@@ -14070,7 +14086,7 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>hecho:zanahorias, dias_desde:zanahorias:28, estudio:ana&gt;=30</t>
+          <t>quedarse, hecho:zanahorias, dias_desde:zanahorias:28, estudio:ana&gt;=30</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -14095,7 +14111,11 @@
           <t>Leer un libro de principio a fin</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr"/>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>quedarse</t>
+        </is>
+      </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Diana presta libros. Un buen rincón: la silla junto a la ventana de la cocina.</t>
@@ -14118,7 +14138,11 @@
           <t>Escribir una carta y mandarla</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr"/>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>quedarse</t>
+        </is>
+      </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
           <t>Se escribe en el escritorio de su pieza; el correo está en la tienda de Lawson.</t>
@@ -14245,7 +14269,11 @@
           <t>Adornar su sombrero con flores</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr"/>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>quedarse</t>
+        </is>
+      </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Con un ramo de la huerta (Marilla no lo va a aprobar).</t>
@@ -14295,7 +14323,11 @@
           <t>Patinar en el lago helado</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr"/>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>quedarse</t>
+        </is>
+      </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Solo en invierno.</t>
@@ -14318,7 +14350,11 @@
           <t>Tirarse en trineo colina abajo</t>
         </is>
       </c>
-      <c r="D29" s="8" t="inlineStr"/>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>quedarse</t>
+        </is>
+      </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
           <t>Solo en invierno, en la colina.</t>
@@ -14341,7 +14377,11 @@
           <t>Teñirse el pelo de negro azabache</t>
         </is>
       </c>
-      <c r="D30" s="8" t="inlineStr"/>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>quedarse</t>
+        </is>
+      </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
           <t>El buhonero vende un tinte que promete maravillas… y acepta huevos.</t>
@@ -31813,7 +31853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31856,109 +31896,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>incoherencia</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>lo que supone que Ana se queda, cuando ya se queda</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>Tillie Boulter</t>
-        </is>
-      </c>
-      <c r="D2" s="8" t="inlineStr">
-        <is>
-          <t>frase</t>
-        </is>
-      </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>día: 1 · estación: primavera · hora: 6:00 · Ana en: el patio de Tejas Verdes · conoce a Tillie Boulter: sí</t>
-        </is>
-      </c>
-      <c r="F2" s="11" t="inlineStr">
-        <is>
-          <t>«Encontré un nido de petirrojos detrás de la escuela. ¡No le digas a nadie!» exige hecho:se_queda</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>incoherencia</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>lo que supone que Ana se queda, cuando ya se queda</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>el reverendo Allan</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>frase</t>
-        </is>
-      </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>día: 1 · estación: primavera · hora: 6:00 · Ana en: el patio de Tejas Verdes · conoce a el reverendo Allan: sí</t>
-        </is>
-      </c>
-      <c r="F3" s="11" t="inlineStr">
-        <is>
-          <t>«Que Dios te bendiga, Ana. ¿Te veremos el domingo en la escuela dominical?» exige hecho:se_queda</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>incoherencia</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>lo que supone que Ana se queda, cuando ya se queda</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>el Sr. Bell</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>frase</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>día: 1 · estación: primavera · hora: 6:00 · Ana en: la cocina de Tejas Verdes · conoce a el Sr. Bell: sí</t>
-        </is>
-      </c>
-      <c r="F4" s="11" t="inlineStr">
-        <is>
-          <t>«Te esperamos el domingo en la escuela dominical, Ana. Y apréndete el versículo.» exige hecho:se_queda</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
-  <conditionalFormatting sqref="A2:A4">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>A2="incoherencia"</formula>
-    </cfRule>
-  </conditionalFormatting>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Jugadoras automáticas para los días a prueba (tools/aprueba.js), y lo que encontraron
- Seis estilos (obediente, rebelde, exploradora, fugitiva, encantadora, insoportable), desde la llegada hasta que
  Marilla decide; revisa en lo que se dijo: repeticiones, nombre sin conocerla, su futuro antes de que la acepten,
  comentar dos veces lo mismo, y que la historia termine a tiempo
- Lo que ya comentó de ella (el camisón, la noche), no lo vuelve a comentar ese día (comento:k:x, también en el guion);
  si una escena suya va a comentarlo, la frase suelta le cede el turno
- Nada se repite delante de Ana: saludos de relleno, charlas y encuentros entre vecinos, avisos de la paciencia
- Los niños cuentan una noticia solo si tiene «dice niños:»; una respuesta solo nombra a quien la cuenta
- La noche (hora:20 o más) es lo que se comenta; las horas de una escena no

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VY3w9XmL1TrbHxLtQe81Lv
</commit_message>
<xml_diff>
--- a/planilla/avonlea.xlsx
+++ b/planilla/avonlea.xlsx
@@ -592,7 +592,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generada el 2026-10-16 17:36 desde los datos del juego (node tools/planilla.js).</t>
+          <t>Generada el 2026-10-16 18:42 desde los datos del juego (node tools/planilla.js).</t>
         </is>
       </c>
     </row>
@@ -12004,7 +12004,7 @@
       <c r="B6" s="11" t="inlineStr"/>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>una frase de barry</t>
+          <t>escena camison_barry, una frase de barry</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr"/>
@@ -12850,7 +12850,7 @@
       <c r="B59" s="11" t="inlineStr"/>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>escena lynde_se_entera, una frase de lynde</t>
+          <t>escena lynde_se_entera, escena camison_lynde, una frase de lynde</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr"/>
@@ -45279,7 +45279,7 @@
       </c>
       <c r="H60" s="9" t="inlineStr">
         <is>
-          <t>ana:camison, !donde:ana:tejas, ve:barry, sabe:barry:nina_cuthbert, hora:7-21</t>
+          <t>ana:camison, !donde:ana:tejas, ve:barry, sabe:barry:nina_cuthbert, !comento:barry:ana:camison, hora:7-21</t>
         </is>
       </c>
       <c r="I60" s="9" t="n"/>
@@ -45334,7 +45334,7 @@
       </c>
       <c r="H61" s="9" t="inlineStr">
         <is>
-          <t>ana:camison, !donde:ana:tejas, ve:lynde, sabe:lynde:nina_cuthbert, hora:7-21</t>
+          <t>ana:camison, !donde:ana:tejas, ve:lynde, sabe:lynde:nina_cuthbert, !comento:lynde:ana:camison, hora:7-21</t>
         </is>
       </c>
       <c r="I61" s="9" t="n"/>
@@ -50629,7 +50629,8 @@
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>lynde: ¿Supo lo de los Cuthbert? ¡Pidieron un niño y les llegó una niña! Pelirroja, dicen. Yo siempre dije que eso de traer huérfanos…</t>
+          <t>lynde: ¿Supo lo de los Cuthbert? ¡Pidieron un niño y les llegó una niña! Pelirroja, dicen. Yo siempre dije que eso de traer huérfanos…
+niños: ¿Sabías? ¡En Tejas Verdes hay una niña nueva! Del orfanato. Y es pelirroja, pelirroja como una zanahoria.</t>
         </is>
       </c>
       <c r="J3" s="9" t="n"/>
@@ -50667,7 +50668,11 @@
           <t>¿Supo que la niña de los Cuthbert anda en camisón por las casas? ¡En camisón!</t>
         </is>
       </c>
-      <c r="I4" s="9" t="n"/>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>niños: ¿Sabías que la niña nueva de Tejas Verdes salió en camisón a la calle? ¡En camisón! Mi mamá dice que eso no se hace.</t>
+        </is>
+      </c>
       <c r="J4" s="9" t="inlineStr">
         <is>
           <t>¿Supo? ¡La niña de los Cuthbert anda en camisón por todo Avonlea, y descalza! Con este frío.
@@ -50705,7 +50710,11 @@
           <t>¿Supo que a los Pye se les escapó otra vez el cerdo? Yo siempre lo dije.</t>
         </is>
       </c>
-      <c r="I5" s="9" t="n"/>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>niños: ¡Se les escapó el chancho a los Pye otra vez! Lo vi correr por el camino.</t>
+        </is>
+      </c>
       <c r="J5" s="9" t="n"/>
       <c r="K5" s="9" t="n"/>
     </row>

</xml_diff>

<commit_message>
Los oficios se aprenden de a un día: ordeñar, partir leña, cocinar
- habilidades.txt: «oficio:» (la acción), «rinde:» y «falla:» por nivel, «mal:» (lo que pasa cuando sale mal); cada
  oficio sube como mucho 1 por día de práctica (no basta con hacerlo una vez), con hitos que le dice Matthew o Marilla
- Ordeñar: al principio, la mitad de las veces se derrama o la vaca se va; con los días, nunca, y más leche
- Partir leña: al principio el hacha rebota o se clava; con los días, más atados
- Cocinar en la estufa: al principio se quema o sale dura (el té, siempre); también cuenta como día de práctica
- Para los demás, como siempre; las pruebas de cadenas del libro (auditoría, metas) parten con Ana ya diestra

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VY3w9XmL1TrbHxLtQe81Lv
</commit_message>
<xml_diff>
--- a/planilla/avonlea.xlsx
+++ b/planilla/avonlea.xlsx
@@ -30,7 +30,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Noticias'!$A$1:$K$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Llegadas'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Diálogos'!$A$1:$C$657</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Hechos'!$A$1:$D$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Hechos'!$A$1:$D$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -592,7 +592,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generada el 2026-10-16 22:38 desde los datos del juego (node tools/planilla.js).</t>
+          <t>Generada el 2026-10-17 06:08 desde los datos del juego (node tools/planilla.js).</t>
         </is>
       </c>
     </row>
@@ -12236,7 +12236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D104"/>
+  <dimension ref="A1:D110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -12960,12 +12960,12 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>hito_paciencia_4</t>
+          <t>hito_mano_cocina_2</t>
         </is>
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>habilidad paciencia</t>
+          <t>habilidad mano_cocina</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr"/>
@@ -12974,98 +12974,82 @@
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>inicio_juego</t>
+          <t>hito_mano_cocina_7</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>código</t>
-        </is>
-      </c>
-      <c r="C46" s="11" t="inlineStr">
-        <is>
-          <t>código</t>
-        </is>
-      </c>
+          <t>habilidad mano_cocina</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr"/>
       <c r="D46" s="8" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>invierno</t>
-        </is>
-      </c>
-      <c r="B47" s="11" t="inlineStr"/>
-      <c r="C47" s="11" t="inlineStr">
-        <is>
-          <t>escena banco_lago_atardecer, escena lugar_bosque_manana, escena lugar_puente, escena lugar_lago_niebla, escena lugar_campo_rosado, escena lugar_playa, escena lugar_rio_escuela, escena lugar_granero, escena lugar_iglesia, escena lugar_corral_idlewild</t>
-        </is>
-      </c>
+          <t>hito_mano_leche_3</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>habilidad mano_leche</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr"/>
       <c r="D47" s="8" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>llamada_almuerzo</t>
+          <t>hito_mano_leche_7</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>escena llamar_almuerzo, escena llamar_almuerzo_afuera</t>
-        </is>
-      </c>
-      <c r="C48" s="11" t="inlineStr">
-        <is>
-          <t>escena llamar_almuerzo, escena llamar_almuerzo_afuera</t>
-        </is>
-      </c>
+          <t>habilidad mano_leche</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="inlineStr"/>
       <c r="D48" s="8" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>llegada_tv</t>
+          <t>hito_mano_lena_2</t>
         </is>
       </c>
       <c r="B49" s="11" t="inlineStr">
         <is>
-          <t>escena llegada, escena inicio_llegada</t>
-        </is>
-      </c>
-      <c r="C49" s="11" t="inlineStr">
-        <is>
-          <t>escena primera_noche, escena desayuno_prueba, una frase de vecino, llegadas de diana</t>
-        </is>
-      </c>
+          <t>habilidad mano_lena</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr"/>
       <c r="D49" s="8" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>llegaron</t>
+          <t>hito_mano_lena_5</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>código</t>
-        </is>
-      </c>
-      <c r="C50" s="11" t="inlineStr">
-        <is>
-          <t>escena llegada</t>
-        </is>
-      </c>
+          <t>habilidad mano_lena</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr"/>
       <c r="D50" s="8" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>llego_</t>
+          <t>hito_paciencia_4</t>
         </is>
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>habilidad paciencia</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr"/>
@@ -13074,17 +13058,17 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>llego_allan</t>
+          <t>inicio_juego</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>llegadas</t>
+          <t>código</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>noticia pastor_nuevo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr"/>
@@ -13092,45 +13076,49 @@
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>llego_buhonero</t>
-        </is>
-      </c>
-      <c r="B53" s="11" t="inlineStr">
-        <is>
-          <t>llegadas</t>
-        </is>
-      </c>
-      <c r="C53" s="11" t="inlineStr"/>
+          <t>invierno</t>
+        </is>
+      </c>
+      <c r="B53" s="11" t="inlineStr"/>
+      <c r="C53" s="11" t="inlineStr">
+        <is>
+          <t>escena banco_lago_atardecer, escena lugar_bosque_manana, escena lugar_puente, escena lugar_lago_niebla, escena lugar_campo_rosado, escena lugar_playa, escena lugar_rio_escuela, escena lugar_granero, escena lugar_iglesia, escena lugar_corral_idlewild</t>
+        </is>
+      </c>
       <c r="D53" s="8" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>llego_diana</t>
+          <t>llamada_almuerzo</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>llegadas</t>
-        </is>
-      </c>
-      <c r="C54" s="11" t="inlineStr"/>
+          <t>escena llamar_almuerzo, escena llamar_almuerzo_afuera</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>escena llamar_almuerzo, escena llamar_almuerzo_afuera</t>
+        </is>
+      </c>
       <c r="D54" s="8" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>llego_gilbert</t>
+          <t>llegada_tv</t>
         </is>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>llegadas</t>
+          <t>escena llegada, escena inicio_llegada</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>escena primera_noche, escena desayuno_prueba, una frase de vecino, llegadas de diana</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr"/>
@@ -13138,17 +13126,17 @@
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>llego_josephine</t>
+          <t>llegaron</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>llegadas</t>
+          <t>código</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>llegadas de phillips</t>
+          <t>escena llegada</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr"/>
@@ -13156,12 +13144,12 @@
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>llego_sraallan</t>
+          <t>llego_</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>llegadas</t>
+          <t>código</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr"/>
@@ -13170,7 +13158,7 @@
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>llego_stacy</t>
+          <t>llego_allan</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
@@ -13180,7 +13168,7 @@
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>noticia pastor_nuevo</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr"/>
@@ -13188,7 +13176,7 @@
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>llego_veraneante</t>
+          <t>llego_buhonero</t>
         </is>
       </c>
       <c r="B59" s="11" t="inlineStr">
@@ -13202,31 +13190,31 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>lynde</t>
-        </is>
-      </c>
-      <c r="B60" s="11" t="inlineStr"/>
-      <c r="C60" s="11" t="inlineStr">
-        <is>
-          <t>escena lynde_se_entera, escena camison_lynde, una frase de lynde</t>
-        </is>
-      </c>
+          <t>llego_diana</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>llegadas</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr"/>
       <c r="D60" s="8" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>lynde_visita</t>
+          <t>llego_gilbert</t>
         </is>
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>escena lynde_visita</t>
+          <t>llegadas</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>una frase de lynde, noticia ana_lengua</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr"/>
@@ -13234,13 +13222,17 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>marilla</t>
-        </is>
-      </c>
-      <c r="B62" s="11" t="inlineStr"/>
+          <t>llego_josephine</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>llegadas</t>
+        </is>
+      </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>escena marilla_sabe_camison, escena marilla_sabe_camison_descalza, escena geranio_sola</t>
+          <t>llegadas de phillips</t>
         </is>
       </c>
       <c r="D62" s="8" t="inlineStr"/>
@@ -13248,31 +13240,31 @@
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>marilla_doblo_ropa</t>
+          <t>llego_sraallan</t>
         </is>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>llegadas</t>
         </is>
       </c>
       <c r="C63" s="11" t="inlineStr"/>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>nadie lo lee</t>
-        </is>
-      </c>
+      <c r="D63" s="8" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>marilla_sabe_camison</t>
-        </is>
-      </c>
-      <c r="B64" s="11" t="inlineStr"/>
+          <t>llego_stacy</t>
+        </is>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>llegadas</t>
+        </is>
+      </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>escena marilla_sabe_camison_descalza</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D64" s="8" t="inlineStr"/>
@@ -13280,35 +13272,27 @@
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>matthew_en_estacion</t>
+          <t>llego_veraneante</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>código</t>
-        </is>
-      </c>
-      <c r="C65" s="11" t="inlineStr">
-        <is>
-          <t>escena estacion</t>
-        </is>
-      </c>
+          <t>llegadas</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="inlineStr"/>
       <c r="D65" s="8" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>matthew_llego_casa</t>
-        </is>
-      </c>
-      <c r="B66" s="11" t="inlineStr">
-        <is>
-          <t>código</t>
-        </is>
-      </c>
+          <t>lynde</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr"/>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>escena tejas_verdes (alternativa)</t>
+          <t>escena lynde_se_entera, escena camison_lynde, una frase de lynde</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr"/>
@@ -13316,13 +13300,17 @@
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>nombra_avenida</t>
-        </is>
-      </c>
-      <c r="B67" s="11" t="inlineStr"/>
+          <t>lynde_visita</t>
+        </is>
+      </c>
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>escena lynde_visita</t>
+        </is>
+      </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>escena conv_matthew_nombres</t>
+          <t>una frase de lynde, noticia ana_lengua</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr"/>
@@ -13330,25 +13318,21 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>nombre_propio_</t>
-        </is>
-      </c>
-      <c r="B68" s="11" t="inlineStr">
-        <is>
-          <t>código</t>
-        </is>
-      </c>
-      <c r="C68" s="11" t="inlineStr"/>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>nadie lo lee</t>
-        </is>
-      </c>
+          <t>marilla</t>
+        </is>
+      </c>
+      <c r="B68" s="11" t="inlineStr"/>
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t>escena marilla_sabe_camison, escena marilla_sabe_camison_descalza, escena geranio_sola</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>nombro_</t>
+          <t>marilla_doblo_ropa</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
@@ -13366,17 +13350,13 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>nombro_avenida</t>
-        </is>
-      </c>
-      <c r="B70" s="11" t="inlineStr">
-        <is>
-          <t>escena nombra_avenida</t>
-        </is>
-      </c>
+          <t>marilla_sabe_camison</t>
+        </is>
+      </c>
+      <c r="B70" s="11" t="inlineStr"/>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>escena conv_matthew_nombres</t>
+          <t>escena marilla_sabe_camison_descalza</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr"/>
@@ -13384,53 +13364,49 @@
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>nombro_burbuja</t>
+          <t>matthew_en_estacion</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>escena conv_diana_nombres</t>
-        </is>
-      </c>
-      <c r="C71" s="11" t="inlineStr"/>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>nadie lo lee</t>
-        </is>
-      </c>
+          <t>código</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="inlineStr">
+        <is>
+          <t>escena estacion</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>nombro_cerezo</t>
+          <t>matthew_llego_casa</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>escena primera_gwin</t>
-        </is>
-      </c>
-      <c r="C72" s="11" t="inlineStr"/>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>nadie lo lee</t>
-        </is>
-      </c>
+          <t>código</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>escena tejas_verdes (alternativa)</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>nombro_geranio</t>
-        </is>
-      </c>
-      <c r="B73" s="11" t="inlineStr">
-        <is>
-          <t>escena primera_geranio, escena geranio_sola</t>
-        </is>
-      </c>
+          <t>nombra_avenida</t>
+        </is>
+      </c>
+      <c r="B73" s="11" t="inlineStr"/>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>escena geranio_sola</t>
+          <t>escena conv_matthew_nombres</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr"/>
@@ -13438,30 +13414,30 @@
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>nombro_lago</t>
+          <t>nombre_propio_</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>escena lago</t>
-        </is>
-      </c>
-      <c r="C74" s="11" t="inlineStr">
-        <is>
-          <t>escena conv_matthew_nombres</t>
-        </is>
-      </c>
-      <c r="D74" s="8" t="inlineStr"/>
+          <t>código</t>
+        </is>
+      </c>
+      <c r="C74" s="11" t="inlineStr"/>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>nadie lo lee</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>nombro_senda</t>
+          <t>nombro_</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>escena conv_diana_nombres</t>
+          <t>código</t>
         </is>
       </c>
       <c r="C75" s="11" t="inlineStr"/>
@@ -13474,17 +13450,17 @@
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>ofendio_lynde</t>
+          <t>nombro_avenida</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
-          <t>escena lynde_visita (una opción)</t>
+          <t>escena nombra_avenida</t>
         </is>
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>escena lynde_disculpa, escena conv_lynde_ventana, escena conv_lynde_pelo, escena conv_lynde_queens, una frase de lynde, noticia ana_lengua</t>
+          <t>escena conv_matthew_nombres</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr"/>
@@ -13492,53 +13468,53 @@
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>pastel_linimento</t>
+          <t>nombro_burbuja</t>
         </is>
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>escena pastel_linimento</t>
-        </is>
-      </c>
-      <c r="C77" s="11" t="inlineStr">
-        <is>
-          <t>meta allan</t>
-        </is>
-      </c>
-      <c r="D77" s="8" t="inlineStr"/>
+          <t>escena conv_diana_nombres</t>
+        </is>
+      </c>
+      <c r="C77" s="11" t="inlineStr"/>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>nadie lo lee</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>perdon_pedido</t>
+          <t>nombro_cerezo</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>escena lynde_perdon_marilla</t>
-        </is>
-      </c>
-      <c r="C78" s="11" t="inlineStr">
-        <is>
-          <t>escena lynde_perdon_marilla</t>
-        </is>
-      </c>
-      <c r="D78" s="8" t="inlineStr"/>
+          <t>escena primera_gwin</t>
+        </is>
+      </c>
+      <c r="C78" s="11" t="inlineStr"/>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>nadie lo lee</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>perdonada</t>
+          <t>nombro_geranio</t>
         </is>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>escena crup_salva</t>
+          <t>escena primera_geranio, escena geranio_sola</t>
         </is>
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>escena ventana_perdonada, escena conv_barry_cordial, una frase de barry, una frase de minnie, una frase de maryjoe, una frase de medico</t>
+          <t>escena geranio_sola</t>
         </is>
       </c>
       <c r="D79" s="8" t="inlineStr"/>
@@ -13546,17 +13522,17 @@
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>pide_amiga</t>
+          <t>nombro_lago</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>escena lago</t>
         </is>
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>escena conv_matthew_nombres</t>
         </is>
       </c>
       <c r="D80" s="8" t="inlineStr"/>
@@ -13564,31 +13540,35 @@
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>primera_bed</t>
-        </is>
-      </c>
-      <c r="B81" s="11" t="inlineStr"/>
-      <c r="C81" s="11" t="inlineStr">
-        <is>
-          <t>escena primera_noche_sube</t>
-        </is>
-      </c>
-      <c r="D81" s="8" t="inlineStr"/>
+          <t>nombro_senda</t>
+        </is>
+      </c>
+      <c r="B81" s="11" t="inlineStr">
+        <is>
+          <t>escena conv_diana_nombres</t>
+        </is>
+      </c>
+      <c r="C81" s="11" t="inlineStr"/>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>nadie lo lee</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>primera_noche</t>
+          <t>ofendio_lynde</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>escena inicio_llegada, escena primera_noche</t>
+          <t>escena lynde_visita (una opción)</t>
         </is>
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>escena primera_noche</t>
+          <t>escena lynde_disculpa, escena conv_lynde_ventana, escena conv_lynde_pelo, escena conv_lynde_queens, una frase de lynde, noticia ana_lengua</t>
         </is>
       </c>
       <c r="D82" s="8" t="inlineStr"/>
@@ -13596,17 +13576,17 @@
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>prohibida</t>
+          <t>pastel_linimento</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>escena prohibida</t>
+          <t>escena pastel_linimento</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>escena barry_no_perdona, escena crup_aviso, escena crup_salva, escena ventana_prohibida, escena lugar_cuesta_prohibida, una frase de diana, una frase de barry</t>
+          <t>meta allan</t>
         </is>
       </c>
       <c r="D83" s="8" t="inlineStr"/>
@@ -13614,17 +13594,17 @@
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>queens</t>
+          <t>perdon_pedido</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>escena examen_primera, escena examen_entra</t>
+          <t>escena lynde_perdon_marilla</t>
         </is>
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>escena ventana_queens, escena faro_queens</t>
+          <t>escena lynde_perdon_marilla</t>
         </is>
       </c>
       <c r="D84" s="8" t="inlineStr"/>
@@ -13632,35 +13612,35 @@
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t>queens_primera</t>
+          <t>perdonada</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>escena examen_primera</t>
-        </is>
-      </c>
-      <c r="C85" s="11" t="inlineStr"/>
-      <c r="D85" s="8" t="inlineStr">
-        <is>
-          <t>nadie lo lee</t>
-        </is>
-      </c>
+          <t>escena crup_salva</t>
+        </is>
+      </c>
+      <c r="C85" s="11" t="inlineStr">
+        <is>
+          <t>escena ventana_perdonada, escena conv_barry_cordial, una frase de barry, una frase de minnie, una frase de maryjoe, una frase de medico</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t>quiere_amiga</t>
+          <t>pide_amiga</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>escena quiere_amiga</t>
+          <t>código</t>
         </is>
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>escena barry_recibe, meta conocer_diana (pista)</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D86" s="8" t="inlineStr"/>
@@ -13668,17 +13648,13 @@
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t>rachel_en_casa_bell</t>
-        </is>
-      </c>
-      <c r="B87" s="11" t="inlineStr">
-        <is>
-          <t>código</t>
-        </is>
-      </c>
+          <t>primera_bed</t>
+        </is>
+      </c>
+      <c r="B87" s="11" t="inlineStr"/>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>escena rachel_bell</t>
+          <t>escena primera_noche_sube</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr"/>
@@ -13686,17 +13662,17 @@
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t>rachel_llego_tejas_verdes</t>
+          <t>primera_noche</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>escena inicio_llegada, escena primera_noche</t>
         </is>
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>escena rachel_marilla</t>
+          <t>escena primera_noche</t>
         </is>
       </c>
       <c r="D88" s="8" t="inlineStr"/>
@@ -13704,17 +13680,17 @@
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t>rachel_lo_sabe</t>
+          <t>prohibida</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>escena rachel_marilla</t>
+          <t>escena prohibida</t>
         </is>
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>escena barry_no_perdona, escena crup_aviso, escena crup_salva, escena ventana_prohibida, escena lugar_cuesta_prohibida, una frase de diana, una frase de barry</t>
         </is>
       </c>
       <c r="D89" s="8" t="inlineStr"/>
@@ -13722,17 +13698,17 @@
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t>ropa_arrugada</t>
+          <t>queens</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>escena examen_primera, escena examen_entra</t>
         </is>
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>una frase de marilla</t>
+          <t>escena ventana_queens, escena faro_queens</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr"/>
@@ -13740,35 +13716,35 @@
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t>ropa_ordenada</t>
+          <t>queens_primera</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>código</t>
-        </is>
-      </c>
-      <c r="C91" s="11" t="inlineStr">
-        <is>
-          <t>una frase de marilla, código</t>
-        </is>
-      </c>
-      <c r="D91" s="8" t="inlineStr"/>
+          <t>escena examen_primera</t>
+        </is>
+      </c>
+      <c r="C91" s="11" t="inlineStr"/>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>nadie lo lee</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t>ropa_tirada_otra</t>
+          <t>quiere_amiga</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>escena quiere_amiga</t>
         </is>
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>escena falta_ropa (una opción), código</t>
+          <t>escena barry_recibe, meta conocer_diana (pista)</t>
         </is>
       </c>
       <c r="D92" s="8" t="inlineStr"/>
@@ -13776,7 +13752,7 @@
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>se_fue_</t>
+          <t>rachel_en_casa_bell</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
@@ -13784,37 +13760,45 @@
           <t>código</t>
         </is>
       </c>
-      <c r="C93" s="11" t="inlineStr"/>
+      <c r="C93" s="11" t="inlineStr">
+        <is>
+          <t>escena rachel_bell</t>
+        </is>
+      </c>
       <c r="D93" s="8" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t>se_fue_buhonero</t>
+          <t>rachel_llego_tejas_verdes</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>llegadas</t>
-        </is>
-      </c>
-      <c r="C94" s="11" t="inlineStr"/>
+          <t>código</t>
+        </is>
+      </c>
+      <c r="C94" s="11" t="inlineStr">
+        <is>
+          <t>escena rachel_marilla</t>
+        </is>
+      </c>
       <c r="D94" s="8" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t>se_fue_josephine</t>
+          <t>rachel_lo_sabe</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>llegadas</t>
+          <t>escena rachel_marilla</t>
         </is>
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>llegadas de allan, llegadas de sraallan</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D95" s="8" t="inlineStr"/>
@@ -13822,17 +13806,17 @@
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t>se_fue_phillips</t>
+          <t>ropa_arrugada</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>llegadas</t>
+          <t>código</t>
         </is>
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>noticia se_va_phillips, llegadas de prissy, llegadas de stacy</t>
+          <t>una frase de marilla</t>
         </is>
       </c>
       <c r="D96" s="8" t="inlineStr"/>
@@ -13840,73 +13824,81 @@
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t>se_fue_prissy</t>
+          <t>ropa_ordenada</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>llegadas</t>
-        </is>
-      </c>
-      <c r="C97" s="11" t="inlineStr"/>
+          <t>código</t>
+        </is>
+      </c>
+      <c r="C97" s="11" t="inlineStr">
+        <is>
+          <t>una frase de marilla, código</t>
+        </is>
+      </c>
       <c r="D97" s="8" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t>se_fue_veraneante</t>
+          <t>ropa_tirada_otra</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>llegadas</t>
-        </is>
-      </c>
-      <c r="C98" s="11" t="inlineStr"/>
+          <t>código</t>
+        </is>
+      </c>
+      <c r="C98" s="11" t="inlineStr">
+        <is>
+          <t>escena falta_ropa (una opción), código</t>
+        </is>
+      </c>
       <c r="D98" s="8" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t>se_queda</t>
+          <t>se_fue_</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>escena se_queda</t>
-        </is>
-      </c>
-      <c r="C99" s="11" t="inlineStr">
-        <is>
-          <t>escena lynde_visita, escena ventana_se_queda, escena espejo_tejas_verdes, escena armario_vestidos, escena lugar_camino_blanco_flor, escena lugar_primera_nieve, escena conv_marilla_por_que, un comentario de espejo, una frase de matthew, una frase de marilla, una frase de lynde, una frase de tillie, una frase de allan, una frase de srbell, meta conocer_diana</t>
-        </is>
-      </c>
+          <t>código</t>
+        </is>
+      </c>
+      <c r="C99" s="11" t="inlineStr"/>
       <c r="D99" s="8" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t>undefined</t>
-        </is>
-      </c>
-      <c r="B100" s="11" t="inlineStr"/>
-      <c r="C100" s="11" t="inlineStr">
-        <is>
-          <t>escena primera_noche, un comentario de sueno_1, un comentario de sueno_2</t>
-        </is>
-      </c>
+          <t>se_fue_buhonero</t>
+        </is>
+      </c>
+      <c r="B100" s="11" t="inlineStr">
+        <is>
+          <t>llegadas</t>
+        </is>
+      </c>
+      <c r="C100" s="11" t="inlineStr"/>
       <c r="D100" s="8" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t>verano</t>
-        </is>
-      </c>
-      <c r="B101" s="11" t="inlineStr"/>
+          <t>se_fue_josephine</t>
+        </is>
+      </c>
+      <c r="B101" s="11" t="inlineStr">
+        <is>
+          <t>llegadas</t>
+        </is>
+      </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>una frase de phillips</t>
+          <t>llegadas de allan, llegadas de sraallan</t>
         </is>
       </c>
       <c r="D101" s="8" t="inlineStr"/>
@@ -13914,13 +13906,17 @@
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B102" s="11" t="inlineStr"/>
+          <t>se_fue_phillips</t>
+        </is>
+      </c>
+      <c r="B102" s="11" t="inlineStr">
+        <is>
+          <t>llegadas</t>
+        </is>
+      </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>noticia se_va_phillips, llegadas de prissy, llegadas de stacy</t>
         </is>
       </c>
       <c r="D102" s="8" t="inlineStr"/>
@@ -13928,39 +13924,127 @@
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t>zanahorias</t>
+          <t>se_fue_prissy</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>escena zanahorias</t>
-        </is>
-      </c>
-      <c r="C103" s="11" t="inlineStr">
-        <is>
-          <t>escena ventana_zanahorias, escena espejo_zanahorias, escena pizarra_zanahorias, escena pupitre_gilbert, escena conv_marilla_john, escena conv_diana_gilbert, un comentario de pupitre, un comentario de pizarra, una frase de gilbert, meta paces</t>
-        </is>
-      </c>
+          <t>llegadas</t>
+        </is>
+      </c>
+      <c r="C103" s="11" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
         <is>
+          <t>se_fue_veraneante</t>
+        </is>
+      </c>
+      <c r="B104" s="11" t="inlineStr">
+        <is>
+          <t>llegadas</t>
+        </is>
+      </c>
+      <c r="C104" s="11" t="inlineStr"/>
+      <c r="D104" s="8" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>se_queda</t>
+        </is>
+      </c>
+      <c r="B105" s="11" t="inlineStr">
+        <is>
+          <t>escena se_queda</t>
+        </is>
+      </c>
+      <c r="C105" s="11" t="inlineStr">
+        <is>
+          <t>escena lynde_visita, escena ventana_se_queda, escena espejo_tejas_verdes, escena armario_vestidos, escena lugar_camino_blanco_flor, escena lugar_primera_nieve, escena conv_marilla_por_que, un comentario de espejo, una frase de matthew, una frase de marilla, una frase de lynde, una frase de tillie, una frase de allan, una frase de srbell, meta conocer_diana</t>
+        </is>
+      </c>
+      <c r="D105" s="8" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t>undefined</t>
+        </is>
+      </c>
+      <c r="B106" s="11" t="inlineStr"/>
+      <c r="C106" s="11" t="inlineStr">
+        <is>
+          <t>escena primera_noche, un comentario de sueno_1, un comentario de sueno_2</t>
+        </is>
+      </c>
+      <c r="D106" s="8" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t>verano</t>
+        </is>
+      </c>
+      <c r="B107" s="11" t="inlineStr"/>
+      <c r="C107" s="11" t="inlineStr">
+        <is>
+          <t>una frase de phillips</t>
+        </is>
+      </c>
+      <c r="D107" s="8" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B108" s="11" t="inlineStr"/>
+      <c r="C108" s="11" t="inlineStr">
+        <is>
+          <t>código</t>
+        </is>
+      </c>
+      <c r="D108" s="8" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="8" t="inlineStr">
+        <is>
+          <t>zanahorias</t>
+        </is>
+      </c>
+      <c r="B109" s="11" t="inlineStr">
+        <is>
+          <t>escena zanahorias</t>
+        </is>
+      </c>
+      <c r="C109" s="11" t="inlineStr">
+        <is>
+          <t>escena ventana_zanahorias, escena espejo_zanahorias, escena pizarra_zanahorias, escena pupitre_gilbert, escena conv_marilla_john, escena conv_diana_gilbert, un comentario de pupitre, un comentario de pizarra, una frase de gilbert, meta paces</t>
+        </is>
+      </c>
+      <c r="D109" s="8" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
           <t>{k}</t>
         </is>
       </c>
-      <c r="B104" s="11" t="inlineStr"/>
-      <c r="C104" s="11" t="inlineStr">
+      <c r="B110" s="11" t="inlineStr"/>
+      <c r="C110" s="11" t="inlineStr">
         <is>
           <t>una frase de niños</t>
         </is>
       </c>
-      <c r="D104" s="8" t="inlineStr"/>
+      <c r="D110" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0"/>
-  <autoFilter ref="A1:D104"/>
-  <conditionalFormatting sqref="D2:D104">
+  <autoFilter ref="A1:D110"/>
+  <conditionalFormatting sqref="D2:D110">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>LEFT(D2,5)="nunca"</formula>
     </cfRule>
@@ -32220,10 +32304,10 @@
       <formula1>=Listas!$C$2:$C$3</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Avonlea" error="No es un hecho ni una meta que exista (¿está bien escrito?)." type="list" errorStyle="warning">
-      <formula1>=Listas!$E$2:$E$119</formula1>
+      <formula1>=Listas!$E$2:$E$125</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Avonlea" error="No es un hecho ni una meta que exista (¿está bien escrito?)." type="list" errorStyle="warning">
-      <formula1>=Listas!$E$2:$E$119</formula1>
+      <formula1>=Listas!$E$2:$E$125</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Avonlea" error="primavera, verano, otoño o invierno." type="list" errorStyle="stop">
       <formula1>=Listas!$D$2:$D$5</formula1>
@@ -39213,7 +39297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E119"/>
+  <dimension ref="A1:E125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39755,7 +39839,7 @@
       </c>
       <c r="E39" s="17" t="inlineStr">
         <is>
-          <t>hito_paciencia_4</t>
+          <t>hito_mano_cocina_2</t>
         </is>
       </c>
     </row>
@@ -39767,7 +39851,7 @@
       </c>
       <c r="E40" s="17" t="inlineStr">
         <is>
-          <t>huerta</t>
+          <t>hito_mano_cocina_7</t>
         </is>
       </c>
     </row>
@@ -39779,7 +39863,7 @@
       </c>
       <c r="E41" s="17" t="inlineStr">
         <is>
-          <t>inicio_juego</t>
+          <t>hito_mano_leche_3</t>
         </is>
       </c>
     </row>
@@ -39791,7 +39875,7 @@
       </c>
       <c r="E42" s="17" t="inlineStr">
         <is>
-          <t>invierno</t>
+          <t>hito_mano_leche_7</t>
         </is>
       </c>
     </row>
@@ -39803,7 +39887,7 @@
       </c>
       <c r="E43" s="17" t="inlineStr">
         <is>
-          <t>josephine</t>
+          <t>hito_mano_lena_2</t>
         </is>
       </c>
     </row>
@@ -39815,7 +39899,7 @@
       </c>
       <c r="E44" s="17" t="inlineStr">
         <is>
-          <t>leido</t>
+          <t>hito_mano_lena_5</t>
         </is>
       </c>
     </row>
@@ -39827,7 +39911,7 @@
       </c>
       <c r="E45" s="17" t="inlineStr">
         <is>
-          <t>llamada_almuerzo</t>
+          <t>hito_paciencia_4</t>
         </is>
       </c>
     </row>
@@ -39839,7 +39923,7 @@
       </c>
       <c r="E46" s="17" t="inlineStr">
         <is>
-          <t>llegada_tv</t>
+          <t>huerta</t>
         </is>
       </c>
     </row>
@@ -39851,7 +39935,7 @@
       </c>
       <c r="E47" s="17" t="inlineStr">
         <is>
-          <t>llegaron</t>
+          <t>inicio_juego</t>
         </is>
       </c>
     </row>
@@ -39863,7 +39947,7 @@
       </c>
       <c r="E48" s="17" t="inlineStr">
         <is>
-          <t>llego_</t>
+          <t>invierno</t>
         </is>
       </c>
     </row>
@@ -39875,7 +39959,7 @@
       </c>
       <c r="E49" s="17" t="inlineStr">
         <is>
-          <t>llego_allan</t>
+          <t>josephine</t>
         </is>
       </c>
     </row>
@@ -39887,7 +39971,7 @@
       </c>
       <c r="E50" s="17" t="inlineStr">
         <is>
-          <t>llego_buhonero</t>
+          <t>leido</t>
         </is>
       </c>
     </row>
@@ -39899,7 +39983,7 @@
       </c>
       <c r="E51" s="17" t="inlineStr">
         <is>
-          <t>llego_diana</t>
+          <t>llamada_almuerzo</t>
         </is>
       </c>
     </row>
@@ -39911,7 +39995,7 @@
       </c>
       <c r="E52" s="17" t="inlineStr">
         <is>
-          <t>llego_gilbert</t>
+          <t>llegada_tv</t>
         </is>
       </c>
     </row>
@@ -39923,7 +40007,7 @@
       </c>
       <c r="E53" s="17" t="inlineStr">
         <is>
-          <t>llego_josephine</t>
+          <t>llegaron</t>
         </is>
       </c>
     </row>
@@ -39935,7 +40019,7 @@
       </c>
       <c r="E54" s="17" t="inlineStr">
         <is>
-          <t>llego_sraallan</t>
+          <t>llego_</t>
         </is>
       </c>
     </row>
@@ -39947,7 +40031,7 @@
       </c>
       <c r="E55" s="17" t="inlineStr">
         <is>
-          <t>llego_stacy</t>
+          <t>llego_allan</t>
         </is>
       </c>
     </row>
@@ -39959,7 +40043,7 @@
       </c>
       <c r="E56" s="17" t="inlineStr">
         <is>
-          <t>llego_veraneante</t>
+          <t>llego_buhonero</t>
         </is>
       </c>
     </row>
@@ -39971,439 +40055,481 @@
       </c>
       <c r="E57" s="17" t="inlineStr">
         <is>
-          <t>lynde</t>
+          <t>llego_diana</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="E58" s="17" t="inlineStr">
         <is>
-          <t>lynde_visita</t>
+          <t>llego_gilbert</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="E59" s="17" t="inlineStr">
         <is>
-          <t>marilla</t>
+          <t>llego_josephine</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="E60" s="17" t="inlineStr">
         <is>
-          <t>marilla_doblo_ropa</t>
+          <t>llego_sraallan</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="E61" s="17" t="inlineStr">
         <is>
-          <t>marilla_sabe_camison</t>
+          <t>llego_stacy</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="E62" s="17" t="inlineStr">
         <is>
-          <t>matthew_en_estacion</t>
+          <t>llego_veraneante</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="E63" s="17" t="inlineStr">
         <is>
-          <t>matthew_llego_casa</t>
+          <t>lynde</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="E64" s="17" t="inlineStr">
         <is>
-          <t>nombra_avenida</t>
+          <t>lynde_visita</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="E65" s="17" t="inlineStr">
         <is>
-          <t>nombre_propio_</t>
+          <t>marilla</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="E66" s="17" t="inlineStr">
         <is>
-          <t>nombres</t>
+          <t>marilla_doblo_ropa</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="E67" s="17" t="inlineStr">
         <is>
-          <t>nombro_</t>
+          <t>marilla_sabe_camison</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="E68" s="17" t="inlineStr">
         <is>
-          <t>nombro_avenida</t>
+          <t>matthew_en_estacion</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="E69" s="17" t="inlineStr">
         <is>
-          <t>nombro_burbuja</t>
+          <t>matthew_llego_casa</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="E70" s="17" t="inlineStr">
         <is>
-          <t>nombro_cerezo</t>
+          <t>nombra_avenida</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="E71" s="17" t="inlineStr">
         <is>
-          <t>nombro_geranio</t>
+          <t>nombre_propio_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="E72" s="17" t="inlineStr">
         <is>
-          <t>nombro_lago</t>
+          <t>nombres</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="E73" s="17" t="inlineStr">
         <is>
-          <t>nombro_senda</t>
+          <t>nombro_</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="E74" s="17" t="inlineStr">
         <is>
-          <t>ofendio_lynde</t>
+          <t>nombro_avenida</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="E75" s="17" t="inlineStr">
         <is>
-          <t>paces</t>
+          <t>nombro_burbuja</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="E76" s="17" t="inlineStr">
         <is>
-          <t>pastel_linimento</t>
+          <t>nombro_cerezo</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="E77" s="17" t="inlineStr">
         <is>
-          <t>patinar</t>
+          <t>nombro_geranio</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="E78" s="17" t="inlineStr">
         <is>
-          <t>pelo_corto</t>
+          <t>nombro_lago</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="E79" s="17" t="inlineStr">
         <is>
-          <t>perdon_barry</t>
+          <t>nombro_senda</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="E80" s="17" t="inlineStr">
         <is>
-          <t>perdon_pedido</t>
+          <t>ofendio_lynde</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="E81" s="17" t="inlineStr">
         <is>
-          <t>perdonada</t>
+          <t>paces</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="E82" s="17" t="inlineStr">
         <is>
-          <t>picnic</t>
+          <t>pastel_linimento</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="E83" s="17" t="inlineStr">
         <is>
-          <t>pide_amiga</t>
+          <t>patinar</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="E84" s="17" t="inlineStr">
         <is>
-          <t>primera_bed</t>
+          <t>pelo_corto</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="E85" s="17" t="inlineStr">
         <is>
-          <t>primera_noche</t>
+          <t>perdon_barry</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="E86" s="17" t="inlineStr">
         <is>
-          <t>prohibida</t>
+          <t>perdon_pedido</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="E87" s="17" t="inlineStr">
         <is>
-          <t>quedarse</t>
+          <t>perdonada</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="E88" s="17" t="inlineStr">
         <is>
-          <t>queens</t>
+          <t>picnic</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="E89" s="17" t="inlineStr">
         <is>
-          <t>queens_primera</t>
+          <t>pide_amiga</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="E90" s="17" t="inlineStr">
         <is>
-          <t>quehaceres</t>
+          <t>primera_bed</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="E91" s="17" t="inlineStr">
         <is>
-          <t>quiere_amiga</t>
+          <t>primera_noche</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="E92" s="17" t="inlineStr">
         <is>
-          <t>rachel_en_casa_bell</t>
+          <t>prohibida</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="E93" s="17" t="inlineStr">
         <is>
-          <t>rachel_llego_tejas_verdes</t>
+          <t>quedarse</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="E94" s="17" t="inlineStr">
         <is>
-          <t>rachel_lo_sabe</t>
+          <t>queens</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="E95" s="17" t="inlineStr">
         <is>
-          <t>recito</t>
+          <t>queens_primera</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="E96" s="17" t="inlineStr">
         <is>
-          <t>regalo</t>
+          <t>quehaceres</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="E97" s="17" t="inlineStr">
         <is>
-          <t>remo</t>
+          <t>quiere_amiga</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="E98" s="17" t="inlineStr">
         <is>
-          <t>rezo</t>
+          <t>rachel_en_casa_bell</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="E99" s="17" t="inlineStr">
         <is>
-          <t>ropa_arrugada</t>
+          <t>rachel_llego_tejas_verdes</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="E100" s="17" t="inlineStr">
         <is>
-          <t>ropa_ordenada</t>
+          <t>rachel_lo_sabe</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="E101" s="17" t="inlineStr">
         <is>
-          <t>ropa_tirada_otra</t>
+          <t>recito</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="E102" s="17" t="inlineStr">
         <is>
-          <t>sala</t>
+          <t>regalo</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="E103" s="17" t="inlineStr">
         <is>
-          <t>se_fue_</t>
+          <t>remo</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="E104" s="17" t="inlineStr">
         <is>
-          <t>se_fue_buhonero</t>
+          <t>rezo</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="E105" s="17" t="inlineStr">
         <is>
-          <t>se_fue_josephine</t>
+          <t>ropa_arrugada</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="E106" s="17" t="inlineStr">
         <is>
-          <t>se_fue_phillips</t>
+          <t>ropa_ordenada</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="E107" s="17" t="inlineStr">
         <is>
-          <t>se_fue_prissy</t>
+          <t>ropa_tirada_otra</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="E108" s="17" t="inlineStr">
         <is>
-          <t>se_fue_veraneante</t>
+          <t>sala</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="E109" s="17" t="inlineStr">
         <is>
-          <t>se_queda</t>
+          <t>se_fue_</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="E110" s="17" t="inlineStr">
         <is>
-          <t>sombrero</t>
+          <t>se_fue_buhonero</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="E111" s="17" t="inlineStr">
         <is>
-          <t>te_diana</t>
+          <t>se_fue_josephine</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="E112" s="17" t="inlineStr">
         <is>
-          <t>techo</t>
+          <t>se_fue_phillips</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="E113" s="17" t="inlineStr">
         <is>
-          <t>tinte</t>
+          <t>se_fue_prissy</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="E114" s="17" t="inlineStr">
         <is>
-          <t>trineo</t>
+          <t>se_fue_veraneante</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="E115" s="17" t="inlineStr">
         <is>
-          <t>undefined</t>
+          <t>se_queda</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="E116" s="17" t="inlineStr">
         <is>
-          <t>verano</t>
+          <t>sombrero</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="E117" s="17" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>te_diana</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="E118" s="17" t="inlineStr">
         <is>
-          <t>zanahorias</t>
+          <t>techo</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="E119" s="17" t="inlineStr">
+        <is>
+          <t>tinte</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="E120" s="17" t="inlineStr">
+        <is>
+          <t>trineo</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="E121" s="17" t="inlineStr">
+        <is>
+          <t>undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="E122" s="17" t="inlineStr">
+        <is>
+          <t>verano</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="E123" s="17" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="E124" s="17" t="inlineStr">
+        <is>
+          <t>zanahorias</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="E125" s="17" t="inlineStr">
         <is>
           <t>{k}</t>
         </is>

</xml_diff>

<commit_message>
Historia: acciones agrupadas por tipo y colapsadas; la cama la primera noche pasa sola
- «sola» en una escena de una línea: pasa sin tocar la cosa, apenas se cumplen
  sus condiciones y Ana está donde dice «en:» (cama_1, la primera noche, en su
  pieza); el juego lo lee del guion en vez del código.
- El comodín de una línea, solo cuando la línea ya empezó (la primera vez es
  el paso 1, o nada).
- Historia en fichas: lo que se puede hacer, agrupado por tipo de acción
  (tocar cosas, pasar por lugares, hablar, escribir…), colapsado; «Irse a
  dormir» de noche.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VY3w9XmL1TrbHxLtQe81Lv
</commit_message>
<xml_diff>
--- a/planilla/avonlea.xlsx
+++ b/planilla/avonlea.xlsx
@@ -592,7 +592,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generada el 2026-10-25 16:29 desde los datos del juego (node tools/planilla.js).</t>
+          <t>Generada el 2026-10-25 17:03 desde los datos del juego (node tools/planilla.js).</t>
         </is>
       </c>
     </row>
@@ -58489,7 +58489,11 @@
           <t>hecho:primera_noche, !hecho:desayuno_prueba, ana_en_tv&lt;se_queda</t>
         </is>
       </c>
-      <c r="I147" s="9" t="n"/>
+      <c r="I147" s="9" t="inlineStr">
+        <is>
+          <t>ana=ga</t>
+        </is>
+      </c>
       <c r="J147" s="9" t="inlineStr">
         <is>
           <t>marilla</t>
@@ -58502,7 +58506,8 @@
         <is>
           <t>resumen: Ana en la pieza del alero, la primera noche: llora hasta dormirse.
 objeto: bed
-paso: 1</t>
+paso: 1
+sola: sí</t>
         </is>
       </c>
       <c r="O147" s="22" t="inlineStr">

</xml_diff>